<commit_message>
adding a historic daily timing plot
of marked vs unmarked fish
</commit_message>
<xml_diff>
--- a/End-of-season Historic escapement files/Daily Totals by Age 2025.xlsx
+++ b/End-of-season Historic escapement files/Daily Totals by Age 2025.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://hupacasath-my.sharepoint.com/personal/graham_hupacasath_ca/Documents/Documents/Graham DOCS/Escapement/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="121" documentId="8_{439EBB09-C0EF-4C9F-A8FE-AAE85C994023}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{82C7A09F-D56A-4FC0-81CC-7160F4F2C029}"/>
+  <xr:revisionPtr revIDLastSave="131" documentId="8_{439EBB09-C0EF-4C9F-A8FE-AAE85C994023}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{687E7163-ED86-41AD-8849-7D36F549A4DB}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="34680" yWindow="45" windowWidth="15810" windowHeight="15435" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sproat" sheetId="1" r:id="rId1"/>
@@ -7767,31 +7767,31 @@
         <v>45893</v>
       </c>
       <c r="B155" s="1">
-        <v>248</v>
+        <v>234</v>
       </c>
       <c r="C155" s="1">
-        <v>188</v>
+        <v>178</v>
       </c>
       <c r="D155" s="1">
-        <v>168.47</v>
+        <v>159.19999999999999</v>
       </c>
       <c r="E155" s="1">
-        <v>158.53</v>
+        <v>149.80000000000001</v>
       </c>
       <c r="F155" s="1">
-        <v>19.84</v>
+        <v>18.75</v>
       </c>
       <c r="G155" s="1">
-        <v>69.37</v>
+        <v>65.55</v>
       </c>
       <c r="H155" s="1">
-        <v>9.9</v>
+        <v>9.35</v>
       </c>
       <c r="I155" s="1">
         <v>0</v>
       </c>
       <c r="J155" s="1">
-        <v>9.9</v>
+        <v>9.35</v>
       </c>
       <c r="K155" s="1">
         <v>0</v>
@@ -7805,31 +7805,31 @@
         <v>45894</v>
       </c>
       <c r="B156" s="1">
-        <v>169</v>
+        <v>151</v>
       </c>
       <c r="C156" s="1">
-        <v>128</v>
+        <v>114</v>
       </c>
       <c r="D156" s="1">
-        <v>114.76</v>
+        <v>102.4</v>
       </c>
       <c r="E156" s="1">
-        <v>107.99</v>
+        <v>96.35</v>
       </c>
       <c r="F156" s="1">
-        <v>13.51</v>
+        <v>12.06</v>
       </c>
       <c r="G156" s="1">
-        <v>47.25</v>
+        <v>42.16</v>
       </c>
       <c r="H156" s="1">
-        <v>6.74</v>
+        <v>6.02</v>
       </c>
       <c r="I156" s="1">
         <v>0</v>
       </c>
       <c r="J156" s="1">
-        <v>6.74</v>
+        <v>6.02</v>
       </c>
       <c r="K156" s="1">
         <v>0</v>
@@ -7843,31 +7843,31 @@
         <v>45895</v>
       </c>
       <c r="B157" s="1">
-        <v>87</v>
+        <v>73</v>
       </c>
       <c r="C157" s="1">
-        <v>66</v>
+        <v>55</v>
       </c>
       <c r="D157" s="1">
-        <v>59.12</v>
+        <v>49.46</v>
       </c>
       <c r="E157" s="1">
-        <v>55.63</v>
+        <v>46.54</v>
       </c>
       <c r="F157" s="1">
-        <v>6.96</v>
+        <v>5.82</v>
       </c>
       <c r="G157" s="1">
-        <v>24.34</v>
+        <v>20.36</v>
       </c>
       <c r="H157" s="1">
-        <v>3.47</v>
+        <v>2.91</v>
       </c>
       <c r="I157" s="1">
         <v>0</v>
       </c>
       <c r="J157" s="1">
-        <v>3.47</v>
+        <v>2.91</v>
       </c>
       <c r="K157" s="1">
         <v>0</v>
@@ -7877,35 +7877,37 @@
       <c r="N157" s="1"/>
     </row>
     <row r="158" spans="1:23" x14ac:dyDescent="0.25">
-      <c r="A158" s="1"/>
-      <c r="B158" s="17">
-        <v>56637</v>
-      </c>
-      <c r="C158" s="17">
-        <v>46308</v>
-      </c>
-      <c r="D158" s="18">
-        <v>42195.86</v>
-      </c>
-      <c r="E158" s="18">
-        <v>38699.78</v>
-      </c>
-      <c r="F158" s="18">
-        <v>4116.59</v>
-      </c>
-      <c r="G158" s="18">
-        <v>13667.17</v>
-      </c>
-      <c r="H158" s="18">
-        <v>3210.68</v>
-      </c>
-      <c r="I158" s="14">
-        <v>0</v>
-      </c>
-      <c r="J158" s="18">
-        <v>1054.92</v>
-      </c>
-      <c r="K158" s="14">
+      <c r="A158" s="10">
+        <v>45896</v>
+      </c>
+      <c r="B158" s="1">
+        <v>40</v>
+      </c>
+      <c r="C158" s="1">
+        <v>30</v>
+      </c>
+      <c r="D158" s="1">
+        <v>27.05</v>
+      </c>
+      <c r="E158" s="1">
+        <v>25.45</v>
+      </c>
+      <c r="F158" s="1">
+        <v>3.19</v>
+      </c>
+      <c r="G158" s="1">
+        <v>11.14</v>
+      </c>
+      <c r="H158" s="1">
+        <v>1.59</v>
+      </c>
+      <c r="I158" s="1">
+        <v>0</v>
+      </c>
+      <c r="J158" s="1">
+        <v>1.59</v>
+      </c>
+      <c r="K158" s="1">
         <v>0</v>
       </c>
       <c r="L158" s="1"/>
@@ -7913,113 +7915,265 @@
       <c r="N158" s="1"/>
     </row>
     <row r="159" spans="1:23" x14ac:dyDescent="0.25">
-      <c r="A159" s="10"/>
-      <c r="B159" s="1"/>
-      <c r="C159" s="1"/>
-      <c r="D159" s="1"/>
-      <c r="E159" s="1"/>
-      <c r="F159" s="1"/>
-      <c r="G159" s="1"/>
-      <c r="H159" s="1"/>
-      <c r="I159" s="1"/>
-      <c r="J159" s="1"/>
-      <c r="K159" s="1"/>
+      <c r="A159" s="10">
+        <v>45897</v>
+      </c>
+      <c r="B159" s="1">
+        <v>16</v>
+      </c>
+      <c r="C159" s="1">
+        <v>12</v>
+      </c>
+      <c r="D159" s="1">
+        <v>10.82</v>
+      </c>
+      <c r="E159" s="1">
+        <v>10.18</v>
+      </c>
+      <c r="F159" s="1">
+        <v>1.27</v>
+      </c>
+      <c r="G159" s="1">
+        <v>4.45</v>
+      </c>
+      <c r="H159" s="1">
+        <v>0.64</v>
+      </c>
+      <c r="I159" s="1">
+        <v>0</v>
+      </c>
+      <c r="J159" s="1">
+        <v>0.64</v>
+      </c>
+      <c r="K159" s="1">
+        <v>0</v>
+      </c>
       <c r="L159" s="1"/>
       <c r="M159" s="1"/>
       <c r="N159" s="1"/>
     </row>
     <row r="160" spans="1:23" x14ac:dyDescent="0.25">
-      <c r="A160" s="10"/>
-      <c r="B160" s="1"/>
-      <c r="C160" s="1"/>
-      <c r="D160" s="1"/>
-      <c r="E160" s="1"/>
-      <c r="F160" s="1"/>
-      <c r="G160" s="1"/>
-      <c r="H160" s="1"/>
-      <c r="I160" s="1"/>
-      <c r="J160" s="1"/>
-      <c r="K160" s="1"/>
+      <c r="A160" s="10">
+        <v>45898</v>
+      </c>
+      <c r="B160" s="1">
+        <v>24</v>
+      </c>
+      <c r="C160" s="1">
+        <v>19</v>
+      </c>
+      <c r="D160" s="1">
+        <v>16.62</v>
+      </c>
+      <c r="E160" s="1">
+        <v>15.63</v>
+      </c>
+      <c r="F160" s="1">
+        <v>1.96</v>
+      </c>
+      <c r="G160" s="1">
+        <v>6.84</v>
+      </c>
+      <c r="H160" s="1">
+        <v>0.98</v>
+      </c>
+      <c r="I160" s="1">
+        <v>0</v>
+      </c>
+      <c r="J160" s="1">
+        <v>0.98</v>
+      </c>
+      <c r="K160" s="1">
+        <v>0</v>
+      </c>
       <c r="L160" s="1"/>
       <c r="M160" s="1"/>
       <c r="N160" s="1"/>
     </row>
     <row r="161" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A161" s="10"/>
-      <c r="B161" s="1"/>
-      <c r="C161" s="1"/>
-      <c r="D161" s="1"/>
-      <c r="E161" s="1"/>
-      <c r="F161" s="1"/>
-      <c r="G161" s="1"/>
-      <c r="H161" s="1"/>
-      <c r="I161" s="1"/>
-      <c r="J161" s="1"/>
-      <c r="K161" s="1"/>
+      <c r="A161" s="10">
+        <v>45899</v>
+      </c>
+      <c r="B161" s="1">
+        <v>31</v>
+      </c>
+      <c r="C161" s="1">
+        <v>23</v>
+      </c>
+      <c r="D161" s="1">
+        <v>20.87</v>
+      </c>
+      <c r="E161" s="1">
+        <v>19.63</v>
+      </c>
+      <c r="F161" s="1">
+        <v>2.46</v>
+      </c>
+      <c r="G161" s="1">
+        <v>8.59</v>
+      </c>
+      <c r="H161" s="1">
+        <v>1.23</v>
+      </c>
+      <c r="I161" s="1">
+        <v>0</v>
+      </c>
+      <c r="J161" s="1">
+        <v>1.23</v>
+      </c>
+      <c r="K161" s="1">
+        <v>0</v>
+      </c>
       <c r="L161" s="1"/>
       <c r="M161" s="1"/>
       <c r="N161" s="1"/>
     </row>
     <row r="162" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A162" s="10"/>
-      <c r="B162" s="1"/>
-      <c r="C162" s="1"/>
-      <c r="D162" s="1"/>
-      <c r="E162" s="1"/>
-      <c r="F162" s="1"/>
-      <c r="G162" s="1"/>
-      <c r="H162" s="1"/>
-      <c r="I162" s="1"/>
-      <c r="J162" s="1"/>
-      <c r="K162" s="1"/>
+      <c r="A162" s="10">
+        <v>45900</v>
+      </c>
+      <c r="B162" s="1">
+        <v>16</v>
+      </c>
+      <c r="C162" s="1">
+        <v>13</v>
+      </c>
+      <c r="D162" s="1">
+        <v>11.21</v>
+      </c>
+      <c r="E162" s="1">
+        <v>10.54</v>
+      </c>
+      <c r="F162" s="1">
+        <v>1.32</v>
+      </c>
+      <c r="G162" s="1">
+        <v>4.6100000000000003</v>
+      </c>
+      <c r="H162" s="1">
+        <v>0.66</v>
+      </c>
+      <c r="I162" s="1">
+        <v>0</v>
+      </c>
+      <c r="J162" s="1">
+        <v>0.66</v>
+      </c>
+      <c r="K162" s="1">
+        <v>0</v>
+      </c>
       <c r="L162" s="1"/>
       <c r="M162" s="1"/>
       <c r="N162" s="1"/>
     </row>
     <row r="163" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A163" s="10"/>
-      <c r="B163" s="1"/>
-      <c r="C163" s="1"/>
-      <c r="D163" s="1"/>
-      <c r="E163" s="1"/>
-      <c r="F163" s="1"/>
-      <c r="G163" s="1"/>
-      <c r="H163" s="1"/>
-      <c r="I163" s="1"/>
-      <c r="J163" s="1"/>
-      <c r="K163" s="1"/>
+      <c r="A163" s="10">
+        <v>45901</v>
+      </c>
+      <c r="B163" s="1">
+        <v>82</v>
+      </c>
+      <c r="C163" s="1">
+        <v>62</v>
+      </c>
+      <c r="D163" s="1">
+        <v>55.64</v>
+      </c>
+      <c r="E163" s="1">
+        <v>52.36</v>
+      </c>
+      <c r="F163" s="1">
+        <v>6.55</v>
+      </c>
+      <c r="G163" s="1">
+        <v>22.91</v>
+      </c>
+      <c r="H163" s="1">
+        <v>3.27</v>
+      </c>
+      <c r="I163" s="1">
+        <v>0</v>
+      </c>
+      <c r="J163" s="1">
+        <v>3.27</v>
+      </c>
+      <c r="K163" s="1">
+        <v>0</v>
+      </c>
       <c r="L163" s="1"/>
       <c r="M163" s="1"/>
       <c r="N163" s="1"/>
     </row>
     <row r="164" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A164" s="10"/>
-      <c r="B164" s="1"/>
-      <c r="C164" s="1"/>
-      <c r="D164" s="1"/>
-      <c r="E164" s="1"/>
-      <c r="F164" s="1"/>
-      <c r="G164" s="1"/>
-      <c r="H164" s="1"/>
-      <c r="I164" s="1"/>
-      <c r="J164" s="1"/>
-      <c r="K164" s="1"/>
+      <c r="A164" s="10">
+        <v>45902</v>
+      </c>
+      <c r="B164" s="1">
+        <v>29</v>
+      </c>
+      <c r="C164" s="1">
+        <v>22</v>
+      </c>
+      <c r="D164" s="1">
+        <v>19.71</v>
+      </c>
+      <c r="E164" s="1">
+        <v>18.54</v>
+      </c>
+      <c r="F164" s="1">
+        <v>2.3199999999999998</v>
+      </c>
+      <c r="G164" s="1">
+        <v>8.11</v>
+      </c>
+      <c r="H164" s="1">
+        <v>1.1599999999999999</v>
+      </c>
+      <c r="I164" s="1">
+        <v>0</v>
+      </c>
+      <c r="J164" s="1">
+        <v>1.1599999999999999</v>
+      </c>
+      <c r="K164" s="1">
+        <v>0</v>
+      </c>
       <c r="L164" s="1"/>
       <c r="M164" s="1"/>
       <c r="N164" s="1"/>
     </row>
     <row r="165" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A165" s="10"/>
-      <c r="B165" s="1"/>
-      <c r="C165" s="1"/>
-      <c r="D165" s="1"/>
-      <c r="E165" s="1"/>
-      <c r="F165" s="1"/>
-      <c r="G165" s="1"/>
-      <c r="H165" s="1"/>
-      <c r="I165" s="1"/>
-      <c r="J165" s="1"/>
-      <c r="K165" s="1"/>
+      <c r="A165" s="1"/>
+      <c r="B165" s="17">
+        <v>56829</v>
+      </c>
+      <c r="C165" s="17">
+        <v>46454</v>
+      </c>
+      <c r="D165" s="18">
+        <v>42326.46</v>
+      </c>
+      <c r="E165" s="18">
+        <v>38822.68</v>
+      </c>
+      <c r="F165" s="18">
+        <v>4131.97</v>
+      </c>
+      <c r="G165" s="18">
+        <v>13720.94</v>
+      </c>
+      <c r="H165" s="18">
+        <v>3218.35</v>
+      </c>
+      <c r="I165" s="14">
+        <v>0</v>
+      </c>
+      <c r="J165" s="18">
+        <v>1062.5899999999999</v>
+      </c>
+      <c r="K165" s="14">
+        <v>0</v>
+      </c>
       <c r="L165" s="1"/>
       <c r="M165" s="1"/>
       <c r="N165" s="1"/>
@@ -14797,31 +14951,31 @@
         <v>45886</v>
       </c>
       <c r="B141" s="15">
-        <v>1018</v>
+        <v>1262</v>
       </c>
       <c r="C141" s="1">
-        <v>432</v>
+        <v>535</v>
       </c>
       <c r="D141" s="1">
-        <v>401.07</v>
+        <v>497.05</v>
       </c>
       <c r="E141" s="1">
-        <v>586.09</v>
+        <v>726.35</v>
       </c>
       <c r="F141" s="1">
-        <v>30.89</v>
+        <v>38.28</v>
       </c>
       <c r="G141" s="1">
-        <v>154.28</v>
+        <v>191.2</v>
       </c>
       <c r="H141" s="1">
-        <v>246.79</v>
+        <v>305.85000000000002</v>
       </c>
       <c r="I141" s="1">
         <v>0</v>
       </c>
       <c r="J141" s="1">
-        <v>30.89</v>
+        <v>38.28</v>
       </c>
       <c r="K141" s="1">
         <v>0</v>
@@ -15153,135 +15307,289 @@
       <c r="L150" s="1"/>
     </row>
     <row r="151" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A151" s="1"/>
-      <c r="B151" s="17">
-        <v>330150</v>
-      </c>
-      <c r="C151" s="17">
-        <v>103513</v>
-      </c>
-      <c r="D151" s="18">
-        <v>89058.14</v>
-      </c>
-      <c r="E151" s="18">
-        <v>198531.79</v>
-      </c>
-      <c r="F151" s="18">
-        <v>14459.57</v>
-      </c>
-      <c r="G151" s="18">
-        <v>64950.97</v>
-      </c>
-      <c r="H151" s="18">
-        <v>63216.07</v>
-      </c>
-      <c r="I151" s="14">
-        <v>0</v>
-      </c>
-      <c r="J151" s="18">
-        <v>3446.46</v>
-      </c>
-      <c r="K151" s="14">
+      <c r="A151" s="10">
+        <v>45896</v>
+      </c>
+      <c r="B151" s="1">
+        <v>314</v>
+      </c>
+      <c r="C151" s="1">
+        <v>133</v>
+      </c>
+      <c r="D151" s="1">
+        <v>123.64</v>
+      </c>
+      <c r="E151" s="1">
+        <v>180.68</v>
+      </c>
+      <c r="F151" s="1">
+        <v>9.52</v>
+      </c>
+      <c r="G151" s="1">
+        <v>47.56</v>
+      </c>
+      <c r="H151" s="1">
+        <v>76.08</v>
+      </c>
+      <c r="I151" s="1">
+        <v>0</v>
+      </c>
+      <c r="J151" s="1">
+        <v>9.52</v>
+      </c>
+      <c r="K151" s="1">
         <v>0</v>
       </c>
       <c r="L151" s="1"/>
     </row>
     <row r="152" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A152" s="10"/>
-      <c r="B152" s="1"/>
-      <c r="C152" s="1"/>
-      <c r="D152" s="1"/>
-      <c r="E152" s="1"/>
-      <c r="F152" s="1"/>
-      <c r="G152" s="1"/>
-      <c r="H152" s="1"/>
-      <c r="I152" s="1"/>
-      <c r="J152" s="1"/>
-      <c r="K152" s="1"/>
+      <c r="A152" s="10">
+        <v>45897</v>
+      </c>
+      <c r="B152" s="1">
+        <v>271</v>
+      </c>
+      <c r="C152" s="1">
+        <v>115</v>
+      </c>
+      <c r="D152" s="1">
+        <v>106.77</v>
+      </c>
+      <c r="E152" s="1">
+        <v>156.02000000000001</v>
+      </c>
+      <c r="F152" s="1">
+        <v>8.2200000000000006</v>
+      </c>
+      <c r="G152" s="1">
+        <v>41.07</v>
+      </c>
+      <c r="H152" s="1">
+        <v>65.7</v>
+      </c>
+      <c r="I152" s="1">
+        <v>0</v>
+      </c>
+      <c r="J152" s="1">
+        <v>8.2200000000000006</v>
+      </c>
+      <c r="K152" s="1">
+        <v>0</v>
+      </c>
       <c r="L152" s="1"/>
     </row>
     <row r="153" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A153" s="10"/>
-      <c r="B153" s="1"/>
-      <c r="C153" s="1"/>
-      <c r="D153" s="1"/>
-      <c r="E153" s="1"/>
-      <c r="F153" s="1"/>
-      <c r="G153" s="1"/>
-      <c r="H153" s="1"/>
-      <c r="I153" s="1"/>
-      <c r="J153" s="1"/>
-      <c r="K153" s="1"/>
+      <c r="A153" s="10">
+        <v>45898</v>
+      </c>
+      <c r="B153" s="1">
+        <v>353</v>
+      </c>
+      <c r="C153" s="1">
+        <v>150</v>
+      </c>
+      <c r="D153" s="1">
+        <v>139.13</v>
+      </c>
+      <c r="E153" s="1">
+        <v>203.31</v>
+      </c>
+      <c r="F153" s="1">
+        <v>10.71</v>
+      </c>
+      <c r="G153" s="1">
+        <v>53.52</v>
+      </c>
+      <c r="H153" s="1">
+        <v>85.61</v>
+      </c>
+      <c r="I153" s="1">
+        <v>0</v>
+      </c>
+      <c r="J153" s="1">
+        <v>10.71</v>
+      </c>
+      <c r="K153" s="1">
+        <v>0</v>
+      </c>
       <c r="L153" s="1"/>
     </row>
     <row r="154" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A154" s="10"/>
-      <c r="B154" s="1"/>
-      <c r="C154" s="1"/>
-      <c r="D154" s="1"/>
-      <c r="E154" s="1"/>
-      <c r="F154" s="1"/>
-      <c r="G154" s="1"/>
-      <c r="H154" s="1"/>
-      <c r="I154" s="1"/>
-      <c r="J154" s="1"/>
-      <c r="K154" s="1"/>
+      <c r="A154" s="10">
+        <v>45899</v>
+      </c>
+      <c r="B154" s="1">
+        <v>496</v>
+      </c>
+      <c r="C154" s="1">
+        <v>211</v>
+      </c>
+      <c r="D154" s="1">
+        <v>195.56</v>
+      </c>
+      <c r="E154" s="1">
+        <v>285.77</v>
+      </c>
+      <c r="F154" s="1">
+        <v>15.06</v>
+      </c>
+      <c r="G154" s="1">
+        <v>75.22</v>
+      </c>
+      <c r="H154" s="1">
+        <v>120.33</v>
+      </c>
+      <c r="I154" s="1">
+        <v>0</v>
+      </c>
+      <c r="J154" s="1">
+        <v>15.06</v>
+      </c>
+      <c r="K154" s="1">
+        <v>0</v>
+      </c>
       <c r="L154" s="1"/>
     </row>
     <row r="155" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A155" s="10"/>
-      <c r="B155" s="1"/>
-      <c r="C155" s="1"/>
-      <c r="D155" s="1"/>
-      <c r="E155" s="1"/>
-      <c r="F155" s="1"/>
-      <c r="G155" s="1"/>
-      <c r="H155" s="1"/>
-      <c r="I155" s="1"/>
-      <c r="J155" s="1"/>
-      <c r="K155" s="1"/>
+      <c r="A155" s="10">
+        <v>45900</v>
+      </c>
+      <c r="B155" s="1">
+        <v>401</v>
+      </c>
+      <c r="C155" s="1">
+        <v>170</v>
+      </c>
+      <c r="D155" s="1">
+        <v>157.94</v>
+      </c>
+      <c r="E155" s="1">
+        <v>230.8</v>
+      </c>
+      <c r="F155" s="1">
+        <v>12.16</v>
+      </c>
+      <c r="G155" s="1">
+        <v>60.75</v>
+      </c>
+      <c r="H155" s="1">
+        <v>97.18</v>
+      </c>
+      <c r="I155" s="1">
+        <v>0</v>
+      </c>
+      <c r="J155" s="1">
+        <v>12.16</v>
+      </c>
+      <c r="K155" s="1">
+        <v>0</v>
+      </c>
       <c r="L155" s="1"/>
     </row>
     <row r="156" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A156" s="10"/>
-      <c r="B156" s="1"/>
-      <c r="C156" s="1"/>
-      <c r="D156" s="1"/>
-      <c r="E156" s="1"/>
-      <c r="F156" s="1"/>
-      <c r="G156" s="1"/>
-      <c r="H156" s="1"/>
-      <c r="I156" s="1"/>
-      <c r="J156" s="1"/>
-      <c r="K156" s="1"/>
+      <c r="A156" s="10">
+        <v>45901</v>
+      </c>
+      <c r="B156" s="1">
+        <v>539</v>
+      </c>
+      <c r="C156" s="1">
+        <v>229</v>
+      </c>
+      <c r="D156" s="1">
+        <v>212.43</v>
+      </c>
+      <c r="E156" s="1">
+        <v>310.43</v>
+      </c>
+      <c r="F156" s="1">
+        <v>16.36</v>
+      </c>
+      <c r="G156" s="1">
+        <v>81.72</v>
+      </c>
+      <c r="H156" s="1">
+        <v>130.71</v>
+      </c>
+      <c r="I156" s="1">
+        <v>0</v>
+      </c>
+      <c r="J156" s="1">
+        <v>16.36</v>
+      </c>
+      <c r="K156" s="1">
+        <v>0</v>
+      </c>
       <c r="L156" s="1"/>
     </row>
     <row r="157" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A157" s="10"/>
-      <c r="B157" s="1"/>
-      <c r="C157" s="1"/>
-      <c r="D157" s="1"/>
-      <c r="E157" s="1"/>
-      <c r="F157" s="1"/>
-      <c r="G157" s="1"/>
-      <c r="H157" s="1"/>
-      <c r="I157" s="1"/>
-      <c r="J157" s="1"/>
-      <c r="K157" s="1"/>
+      <c r="A157" s="10">
+        <v>45902</v>
+      </c>
+      <c r="B157" s="1">
+        <v>191</v>
+      </c>
+      <c r="C157" s="1">
+        <v>81</v>
+      </c>
+      <c r="D157" s="1">
+        <v>75.239999999999995</v>
+      </c>
+      <c r="E157" s="1">
+        <v>109.94</v>
+      </c>
+      <c r="F157" s="1">
+        <v>5.79</v>
+      </c>
+      <c r="G157" s="1">
+        <v>28.94</v>
+      </c>
+      <c r="H157" s="1">
+        <v>46.29</v>
+      </c>
+      <c r="I157" s="1">
+        <v>0</v>
+      </c>
+      <c r="J157" s="1">
+        <v>5.79</v>
+      </c>
+      <c r="K157" s="1">
+        <v>0</v>
+      </c>
       <c r="L157" s="1"/>
     </row>
     <row r="158" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A158" s="10"/>
-      <c r="B158" s="1"/>
-      <c r="C158" s="1"/>
-      <c r="D158" s="1"/>
-      <c r="E158" s="1"/>
-      <c r="F158" s="1"/>
-      <c r="G158" s="1"/>
-      <c r="H158" s="1"/>
-      <c r="I158" s="1"/>
-      <c r="J158" s="1"/>
-      <c r="K158" s="1"/>
+      <c r="A158" s="1"/>
+      <c r="B158" s="17">
+        <v>332959</v>
+      </c>
+      <c r="C158" s="17">
+        <v>104705</v>
+      </c>
+      <c r="D158" s="18">
+        <v>90164.82</v>
+      </c>
+      <c r="E158" s="18">
+        <v>200149</v>
+      </c>
+      <c r="F158" s="18">
+        <v>14544.8</v>
+      </c>
+      <c r="G158" s="18">
+        <v>65376.68</v>
+      </c>
+      <c r="H158" s="18">
+        <v>63897.04</v>
+      </c>
+      <c r="I158" s="14">
+        <v>0</v>
+      </c>
+      <c r="J158" s="18">
+        <v>3531.68</v>
+      </c>
+      <c r="K158" s="14">
+        <v>0</v>
+      </c>
       <c r="L158" s="1"/>
     </row>
     <row r="159" spans="1:12" x14ac:dyDescent="0.25">
@@ -20625,10 +20933,10 @@
         <v>45893</v>
       </c>
       <c r="B154" s="1">
-        <v>262.87</v>
+        <v>248.78</v>
       </c>
       <c r="C154" s="1">
-        <v>16.34</v>
+        <v>15.47</v>
       </c>
       <c r="D154" s="1">
         <v>0</v>
@@ -20654,13 +20962,13 @@
         <v>45894</v>
       </c>
       <c r="B155" s="1">
-        <v>141.65</v>
+        <v>126.46</v>
       </c>
       <c r="C155" s="1">
-        <v>50.39</v>
+        <v>44.99</v>
       </c>
       <c r="D155" s="1">
-        <v>1.36</v>
+        <v>1.22</v>
       </c>
       <c r="E155" s="1">
         <v>0</v>
@@ -20683,10 +20991,10 @@
         <v>45895</v>
       </c>
       <c r="B156" s="1">
-        <v>119.86</v>
+        <v>100.58</v>
       </c>
       <c r="C156" s="1">
-        <v>29.96</v>
+        <v>25.15</v>
       </c>
       <c r="D156" s="1">
         <v>0</v>
@@ -20708,108 +21016,234 @@
       </c>
     </row>
     <row r="157" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A157" s="10"/>
-      <c r="B157" s="14">
-        <v>3975.01</v>
-      </c>
-      <c r="C157" s="14">
-        <v>262.86</v>
-      </c>
-      <c r="D157" s="14">
-        <v>1.36</v>
-      </c>
-      <c r="E157" s="14">
-        <v>0</v>
-      </c>
-      <c r="F157" s="14">
-        <v>0</v>
-      </c>
-      <c r="G157" s="14">
-        <v>1.33</v>
-      </c>
-      <c r="H157" s="14">
-        <v>64.680000000000007</v>
-      </c>
-      <c r="I157" s="14">
-        <v>11.36</v>
+      <c r="A157" s="10">
+        <v>45896</v>
+      </c>
+      <c r="B157" s="1">
+        <v>51.36</v>
+      </c>
+      <c r="C157" s="1">
+        <v>22.47</v>
+      </c>
+      <c r="D157" s="1">
+        <v>0</v>
+      </c>
+      <c r="E157" s="1">
+        <v>0</v>
+      </c>
+      <c r="F157" s="1">
+        <v>0</v>
+      </c>
+      <c r="G157" s="1">
+        <v>0</v>
+      </c>
+      <c r="H157" s="1">
+        <v>0</v>
+      </c>
+      <c r="I157" s="1">
+        <v>0</v>
       </c>
     </row>
     <row r="158" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A158" s="10"/>
-      <c r="B158" s="1"/>
-      <c r="C158" s="1"/>
-      <c r="D158" s="1"/>
-      <c r="E158" s="1"/>
-      <c r="F158" s="1"/>
-      <c r="G158" s="1"/>
-      <c r="H158" s="1"/>
-      <c r="I158" s="1"/>
+      <c r="A158" s="10">
+        <v>45897</v>
+      </c>
+      <c r="B158" s="1">
+        <v>30</v>
+      </c>
+      <c r="C158" s="1">
+        <v>10</v>
+      </c>
+      <c r="D158" s="1">
+        <v>0</v>
+      </c>
+      <c r="E158" s="1">
+        <v>0</v>
+      </c>
+      <c r="F158" s="1">
+        <v>0</v>
+      </c>
+      <c r="G158" s="1">
+        <v>0</v>
+      </c>
+      <c r="H158" s="1">
+        <v>0</v>
+      </c>
+      <c r="I158" s="1">
+        <v>0</v>
+      </c>
     </row>
     <row r="159" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A159" s="10"/>
-      <c r="B159" s="1"/>
-      <c r="C159" s="1"/>
-      <c r="D159" s="1"/>
-      <c r="E159" s="1"/>
-      <c r="F159" s="1"/>
-      <c r="G159" s="1"/>
-      <c r="H159" s="1"/>
-      <c r="I159" s="1"/>
+      <c r="A159" s="10">
+        <v>45898</v>
+      </c>
+      <c r="B159" s="1">
+        <v>27.09</v>
+      </c>
+      <c r="C159" s="1">
+        <v>0</v>
+      </c>
+      <c r="D159" s="1">
+        <v>0</v>
+      </c>
+      <c r="E159" s="1">
+        <v>0</v>
+      </c>
+      <c r="F159" s="1">
+        <v>0</v>
+      </c>
+      <c r="G159" s="1">
+        <v>0</v>
+      </c>
+      <c r="H159" s="1">
+        <v>1.04</v>
+      </c>
+      <c r="I159" s="1">
+        <v>0</v>
+      </c>
     </row>
     <row r="160" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A160" s="10"/>
-      <c r="B160" s="1"/>
-      <c r="C160" s="1"/>
-      <c r="D160" s="1"/>
-      <c r="E160" s="1"/>
-      <c r="F160" s="1"/>
-      <c r="G160" s="1"/>
-      <c r="H160" s="1"/>
-      <c r="I160" s="1"/>
+      <c r="A160" s="10">
+        <v>45899</v>
+      </c>
+      <c r="B160" s="1">
+        <v>80.14</v>
+      </c>
+      <c r="C160" s="1">
+        <v>16.239999999999998</v>
+      </c>
+      <c r="D160" s="1">
+        <v>0</v>
+      </c>
+      <c r="E160" s="1">
+        <v>0</v>
+      </c>
+      <c r="F160" s="1">
+        <v>0</v>
+      </c>
+      <c r="G160" s="1">
+        <v>0</v>
+      </c>
+      <c r="H160" s="1">
+        <v>0</v>
+      </c>
+      <c r="I160" s="1">
+        <v>0</v>
+      </c>
     </row>
     <row r="161" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A161" s="10"/>
-      <c r="B161" s="1"/>
-      <c r="C161" s="1"/>
-      <c r="D161" s="1"/>
-      <c r="E161" s="1"/>
-      <c r="F161" s="1"/>
-      <c r="G161" s="1"/>
-      <c r="H161" s="1"/>
-      <c r="I161" s="1"/>
+      <c r="A161" s="10">
+        <v>45900</v>
+      </c>
+      <c r="B161" s="1">
+        <v>112.37</v>
+      </c>
+      <c r="C161" s="1">
+        <v>13.09</v>
+      </c>
+      <c r="D161" s="1">
+        <v>0</v>
+      </c>
+      <c r="E161" s="1">
+        <v>0</v>
+      </c>
+      <c r="F161" s="1">
+        <v>1.0900000000000001</v>
+      </c>
+      <c r="G161" s="1">
+        <v>0</v>
+      </c>
+      <c r="H161" s="1">
+        <v>0</v>
+      </c>
+      <c r="I161" s="1">
+        <v>0</v>
+      </c>
     </row>
     <row r="162" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A162" s="10"/>
-      <c r="B162" s="1"/>
-      <c r="C162" s="1"/>
-      <c r="D162" s="1"/>
-      <c r="E162" s="1"/>
-      <c r="F162" s="1"/>
-      <c r="G162" s="1"/>
-      <c r="H162" s="1"/>
-      <c r="I162" s="1"/>
+      <c r="A162" s="10">
+        <v>45901</v>
+      </c>
+      <c r="B162" s="1">
+        <v>96.71</v>
+      </c>
+      <c r="C162" s="1">
+        <v>0</v>
+      </c>
+      <c r="D162" s="1">
+        <v>0</v>
+      </c>
+      <c r="E162" s="1">
+        <v>0</v>
+      </c>
+      <c r="F162" s="1">
+        <v>0</v>
+      </c>
+      <c r="G162" s="1">
+        <v>0</v>
+      </c>
+      <c r="H162" s="1">
+        <v>0</v>
+      </c>
+      <c r="I162" s="1">
+        <v>0</v>
+      </c>
     </row>
     <row r="163" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A163" s="10"/>
-      <c r="B163" s="1"/>
-      <c r="C163" s="1"/>
-      <c r="D163" s="1"/>
-      <c r="E163" s="1"/>
-      <c r="F163" s="1"/>
-      <c r="G163" s="1"/>
-      <c r="H163" s="1"/>
-      <c r="I163" s="1"/>
+      <c r="A163" s="10">
+        <v>45902</v>
+      </c>
+      <c r="B163" s="1">
+        <v>128.63999999999999</v>
+      </c>
+      <c r="C163" s="1">
+        <v>75.41</v>
+      </c>
+      <c r="D163" s="1">
+        <v>0</v>
+      </c>
+      <c r="E163" s="1">
+        <v>0</v>
+      </c>
+      <c r="F163" s="1">
+        <v>0</v>
+      </c>
+      <c r="G163" s="1">
+        <v>0</v>
+      </c>
+      <c r="H163" s="1">
+        <v>0</v>
+      </c>
+      <c r="I163" s="1">
+        <v>0</v>
+      </c>
     </row>
     <row r="164" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A164" s="10"/>
-      <c r="B164" s="1"/>
-      <c r="C164" s="1"/>
-      <c r="D164" s="1"/>
-      <c r="E164" s="1"/>
-      <c r="F164" s="1"/>
-      <c r="G164" s="1"/>
-      <c r="H164" s="1"/>
-      <c r="I164" s="1"/>
+      <c r="B164" s="14">
+        <v>4452.76</v>
+      </c>
+      <c r="C164" s="14">
+        <v>388.99</v>
+      </c>
+      <c r="D164" s="14">
+        <v>1.22</v>
+      </c>
+      <c r="E164" s="14">
+        <v>0</v>
+      </c>
+      <c r="F164" s="14">
+        <v>1.0900000000000001</v>
+      </c>
+      <c r="G164" s="14">
+        <v>1.33</v>
+      </c>
+      <c r="H164" s="14">
+        <v>65.72</v>
+      </c>
+      <c r="I164" s="14">
+        <v>11.36</v>
+      </c>
     </row>
     <row r="165" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A165" s="10"/>
@@ -38432,10 +38866,10 @@
         <v>45886</v>
       </c>
       <c r="B140" s="1">
-        <v>48.5</v>
+        <v>28</v>
       </c>
       <c r="C140" s="1">
-        <v>5.5</v>
+        <v>3</v>
       </c>
       <c r="D140" s="1">
         <v>0</v>
@@ -38444,13 +38878,13 @@
         <v>0</v>
       </c>
       <c r="F140" s="1">
-        <v>118.5</v>
+        <v>96</v>
       </c>
       <c r="G140" s="1">
-        <v>12</v>
+        <v>8</v>
       </c>
       <c r="H140" s="1">
-        <v>8.5</v>
+        <v>9</v>
       </c>
       <c r="I140" s="1">
         <v>0</v>
@@ -38460,7 +38894,7 @@
         <v>0</v>
       </c>
       <c r="L140" s="1">
-        <v>1445.5</v>
+        <v>1762</v>
       </c>
       <c r="M140" s="1">
         <v>0</v>
@@ -38469,7 +38903,7 @@
         <v>0</v>
       </c>
       <c r="O140" s="1">
-        <v>3.5</v>
+        <v>35</v>
       </c>
       <c r="P140" s="1">
         <v>0</v>
@@ -38478,16 +38912,16 @@
         <v>0</v>
       </c>
       <c r="R140" s="1">
-        <v>41</v>
+        <v>23</v>
       </c>
       <c r="S140" s="1">
-        <v>7.5</v>
+        <v>5</v>
       </c>
       <c r="T140" s="1">
         <v>0</v>
       </c>
       <c r="U140" s="1">
-        <v>5.5</v>
+        <v>3</v>
       </c>
       <c r="V140" s="1">
         <v>0</v>
@@ -38514,28 +38948,28 @@
         <v>0</v>
       </c>
       <c r="AD140" s="1">
-        <v>106.5</v>
+        <v>90</v>
       </c>
       <c r="AE140" s="1">
-        <v>12</v>
+        <v>6</v>
       </c>
       <c r="AF140" s="1">
         <v>0</v>
       </c>
       <c r="AG140" s="1">
-        <v>4.5</v>
+        <v>0</v>
       </c>
       <c r="AH140" s="1">
-        <v>7.5</v>
+        <v>8</v>
       </c>
       <c r="AI140" s="1">
         <v>0</v>
       </c>
       <c r="AJ140" s="1">
-        <v>6.5</v>
+        <v>6</v>
       </c>
       <c r="AK140" s="1">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="AL140" s="1">
         <v>0</v>
@@ -39628,37 +40062,39 @@
       </c>
     </row>
     <row r="150" spans="1:40" x14ac:dyDescent="0.25">
-      <c r="A150" s="10"/>
-      <c r="B150" s="14">
-        <v>1381.5</v>
-      </c>
-      <c r="C150" s="14">
-        <v>294.5</v>
-      </c>
-      <c r="D150" s="14">
-        <v>0</v>
-      </c>
-      <c r="E150" s="14">
-        <v>0</v>
-      </c>
-      <c r="F150" s="14">
-        <v>3896.5</v>
-      </c>
-      <c r="G150" s="14">
-        <v>690</v>
-      </c>
-      <c r="H150" s="14">
-        <v>869</v>
-      </c>
-      <c r="I150" s="14">
-        <v>16</v>
+      <c r="A150" s="10">
+        <v>45896</v>
+      </c>
+      <c r="B150" s="1">
+        <v>45</v>
+      </c>
+      <c r="C150" s="1">
+        <v>21</v>
+      </c>
+      <c r="D150" s="1">
+        <v>0</v>
+      </c>
+      <c r="E150" s="1">
+        <v>0</v>
+      </c>
+      <c r="F150" s="1">
+        <v>265</v>
+      </c>
+      <c r="G150" s="1">
+        <v>89</v>
+      </c>
+      <c r="H150" s="1">
+        <v>23</v>
+      </c>
+      <c r="I150" s="1">
+        <v>0</v>
       </c>
       <c r="J150" s="1"/>
       <c r="K150" s="1">
         <v>0</v>
       </c>
       <c r="L150" s="1">
-        <v>429968.46</v>
+        <v>438</v>
       </c>
       <c r="M150" s="1">
         <v>0</v>
@@ -39667,7 +40103,7 @@
         <v>0</v>
       </c>
       <c r="O150" s="1">
-        <v>3689.5</v>
+        <v>9</v>
       </c>
       <c r="P150" s="1">
         <v>0</v>
@@ -39676,151 +40112,912 @@
         <v>0</v>
       </c>
       <c r="R150" s="1">
-        <v>1128</v>
+        <v>39</v>
       </c>
       <c r="S150" s="1">
-        <v>253.5</v>
+        <v>6</v>
       </c>
       <c r="T150" s="1">
         <v>0</v>
       </c>
       <c r="U150" s="1">
-        <v>278.5</v>
+        <v>18</v>
       </c>
       <c r="V150" s="1">
+        <v>3</v>
+      </c>
+      <c r="W150" s="1">
+        <v>0</v>
+      </c>
+      <c r="X150" s="1">
+        <v>0</v>
+      </c>
+      <c r="Y150" s="1">
+        <v>0</v>
+      </c>
+      <c r="Z150" s="1">
+        <v>0</v>
+      </c>
+      <c r="AA150" s="1">
+        <v>0</v>
+      </c>
+      <c r="AB150" s="1">
+        <v>0</v>
+      </c>
+      <c r="AC150" s="1">
+        <v>0</v>
+      </c>
+      <c r="AD150" s="1">
+        <v>245</v>
+      </c>
+      <c r="AE150" s="1">
+        <v>20</v>
+      </c>
+      <c r="AF150" s="1">
+        <v>0</v>
+      </c>
+      <c r="AG150" s="1">
+        <v>8</v>
+      </c>
+      <c r="AH150" s="1">
+        <v>81</v>
+      </c>
+      <c r="AI150" s="1">
+        <v>0</v>
+      </c>
+      <c r="AJ150" s="1">
+        <v>21</v>
+      </c>
+      <c r="AK150" s="1">
+        <v>2</v>
+      </c>
+      <c r="AL150" s="1">
+        <v>0</v>
+      </c>
+      <c r="AM150" s="1">
+        <v>0</v>
+      </c>
+      <c r="AN150" s="1">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="151" spans="1:40" x14ac:dyDescent="0.25">
+      <c r="A151" s="10">
+        <v>45897</v>
+      </c>
+      <c r="B151" s="1">
+        <v>31</v>
+      </c>
+      <c r="C151" s="1">
+        <v>23</v>
+      </c>
+      <c r="D151" s="1">
+        <v>0</v>
+      </c>
+      <c r="E151" s="1">
+        <v>0</v>
+      </c>
+      <c r="F151" s="1">
+        <v>140</v>
+      </c>
+      <c r="G151" s="1">
+        <v>121</v>
+      </c>
+      <c r="H151" s="1">
+        <v>14</v>
+      </c>
+      <c r="I151" s="1">
+        <v>0</v>
+      </c>
+      <c r="J151" s="1"/>
+      <c r="K151" s="1">
+        <v>0</v>
+      </c>
+      <c r="L151" s="1">
+        <v>386</v>
+      </c>
+      <c r="M151" s="1">
+        <v>0</v>
+      </c>
+      <c r="N151" s="1">
+        <v>0</v>
+      </c>
+      <c r="O151" s="1">
+        <v>0</v>
+      </c>
+      <c r="P151" s="1">
+        <v>0</v>
+      </c>
+      <c r="Q151" s="1">
+        <v>0</v>
+      </c>
+      <c r="R151" s="1">
+        <v>24</v>
+      </c>
+      <c r="S151" s="1">
+        <v>7</v>
+      </c>
+      <c r="T151" s="1">
+        <v>0</v>
+      </c>
+      <c r="U151" s="1">
+        <v>22</v>
+      </c>
+      <c r="V151" s="1">
+        <v>1</v>
+      </c>
+      <c r="W151" s="1">
+        <v>0</v>
+      </c>
+      <c r="X151" s="1">
+        <v>0</v>
+      </c>
+      <c r="Y151" s="1">
+        <v>0</v>
+      </c>
+      <c r="Z151" s="1">
+        <v>0</v>
+      </c>
+      <c r="AA151" s="1">
+        <v>0</v>
+      </c>
+      <c r="AB151" s="1">
+        <v>0</v>
+      </c>
+      <c r="AC151" s="1">
+        <v>0</v>
+      </c>
+      <c r="AD151" s="1">
+        <v>127</v>
+      </c>
+      <c r="AE151" s="1">
+        <v>13</v>
+      </c>
+      <c r="AF151" s="1">
+        <v>0</v>
+      </c>
+      <c r="AG151" s="1">
+        <v>18</v>
+      </c>
+      <c r="AH151" s="1">
+        <v>103</v>
+      </c>
+      <c r="AI151" s="1">
+        <v>0</v>
+      </c>
+      <c r="AJ151" s="1">
+        <v>9</v>
+      </c>
+      <c r="AK151" s="1">
+        <v>5</v>
+      </c>
+      <c r="AL151" s="1">
+        <v>0</v>
+      </c>
+      <c r="AM151" s="1">
+        <v>0</v>
+      </c>
+      <c r="AN151" s="1">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="152" spans="1:40" x14ac:dyDescent="0.25">
+      <c r="A152" s="10">
+        <v>45898</v>
+      </c>
+      <c r="B152" s="1">
+        <v>36</v>
+      </c>
+      <c r="C152" s="1">
+        <v>25</v>
+      </c>
+      <c r="D152" s="1">
+        <v>0</v>
+      </c>
+      <c r="E152" s="1">
+        <v>0</v>
+      </c>
+      <c r="F152" s="1">
+        <v>107</v>
+      </c>
+      <c r="G152" s="1">
+        <v>130</v>
+      </c>
+      <c r="H152" s="1">
+        <v>10</v>
+      </c>
+      <c r="I152" s="1">
+        <v>0</v>
+      </c>
+      <c r="J152" s="1"/>
+      <c r="K152" s="1">
+        <v>0</v>
+      </c>
+      <c r="L152" s="1">
+        <v>503</v>
+      </c>
+      <c r="M152" s="1">
+        <v>0</v>
+      </c>
+      <c r="N152" s="1">
+        <v>0</v>
+      </c>
+      <c r="O152" s="1">
+        <v>0</v>
+      </c>
+      <c r="P152" s="1">
+        <v>0</v>
+      </c>
+      <c r="Q152" s="1">
+        <v>0</v>
+      </c>
+      <c r="R152" s="1">
+        <v>29</v>
+      </c>
+      <c r="S152" s="1">
+        <v>7</v>
+      </c>
+      <c r="T152" s="1">
+        <v>0</v>
+      </c>
+      <c r="U152" s="1">
+        <v>23</v>
+      </c>
+      <c r="V152" s="1">
+        <v>2</v>
+      </c>
+      <c r="W152" s="1">
+        <v>0</v>
+      </c>
+      <c r="X152" s="1">
+        <v>0</v>
+      </c>
+      <c r="Y152" s="1">
+        <v>0</v>
+      </c>
+      <c r="Z152" s="1">
+        <v>0</v>
+      </c>
+      <c r="AA152" s="1">
+        <v>0</v>
+      </c>
+      <c r="AB152" s="1">
+        <v>0</v>
+      </c>
+      <c r="AC152" s="1">
+        <v>0</v>
+      </c>
+      <c r="AD152" s="1">
+        <v>98</v>
+      </c>
+      <c r="AE152" s="1">
+        <v>9</v>
+      </c>
+      <c r="AF152" s="1">
+        <v>0</v>
+      </c>
+      <c r="AG152" s="1">
+        <v>43</v>
+      </c>
+      <c r="AH152" s="1">
+        <v>87</v>
+      </c>
+      <c r="AI152" s="1">
+        <v>0</v>
+      </c>
+      <c r="AJ152" s="1">
+        <v>9</v>
+      </c>
+      <c r="AK152" s="1">
+        <v>1</v>
+      </c>
+      <c r="AL152" s="1">
+        <v>0</v>
+      </c>
+      <c r="AM152" s="1">
+        <v>0</v>
+      </c>
+      <c r="AN152" s="1">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="153" spans="1:40" x14ac:dyDescent="0.25">
+      <c r="A153" s="10">
+        <v>45899</v>
+      </c>
+      <c r="B153" s="1">
+        <v>100</v>
+      </c>
+      <c r="C153" s="1">
+        <v>57</v>
+      </c>
+      <c r="D153" s="1">
+        <v>0</v>
+      </c>
+      <c r="E153" s="1">
+        <v>0</v>
+      </c>
+      <c r="F153" s="1">
+        <v>153</v>
+      </c>
+      <c r="G153" s="1">
+        <v>190</v>
+      </c>
+      <c r="H153" s="1">
+        <v>13</v>
+      </c>
+      <c r="I153" s="1">
+        <v>0</v>
+      </c>
+      <c r="J153" s="1"/>
+      <c r="K153" s="1">
+        <v>0</v>
+      </c>
+      <c r="L153" s="1">
+        <v>707</v>
+      </c>
+      <c r="M153" s="1">
+        <v>0</v>
+      </c>
+      <c r="N153" s="1">
+        <v>0</v>
+      </c>
+      <c r="O153" s="1">
+        <v>0</v>
+      </c>
+      <c r="P153" s="1">
+        <v>0</v>
+      </c>
+      <c r="Q153" s="1">
+        <v>0</v>
+      </c>
+      <c r="R153" s="1">
+        <v>85</v>
+      </c>
+      <c r="S153" s="1">
+        <v>15</v>
+      </c>
+      <c r="T153" s="1">
+        <v>0</v>
+      </c>
+      <c r="U153" s="1">
+        <v>50</v>
+      </c>
+      <c r="V153" s="1">
+        <v>7</v>
+      </c>
+      <c r="W153" s="1">
+        <v>0</v>
+      </c>
+      <c r="X153" s="1">
+        <v>0</v>
+      </c>
+      <c r="Y153" s="1">
+        <v>0</v>
+      </c>
+      <c r="Z153" s="1">
+        <v>0</v>
+      </c>
+      <c r="AA153" s="1">
+        <v>0</v>
+      </c>
+      <c r="AB153" s="1">
+        <v>0</v>
+      </c>
+      <c r="AC153" s="1">
+        <v>0</v>
+      </c>
+      <c r="AD153" s="1">
+        <v>141</v>
+      </c>
+      <c r="AE153" s="1">
+        <v>12</v>
+      </c>
+      <c r="AF153" s="1">
+        <v>0</v>
+      </c>
+      <c r="AG153" s="1">
+        <v>25</v>
+      </c>
+      <c r="AH153" s="1">
+        <v>165</v>
+      </c>
+      <c r="AI153" s="1">
+        <v>0</v>
+      </c>
+      <c r="AJ153" s="1">
+        <v>11</v>
+      </c>
+      <c r="AK153" s="1">
+        <v>2</v>
+      </c>
+      <c r="AL153" s="1">
+        <v>0</v>
+      </c>
+      <c r="AM153" s="1">
+        <v>0</v>
+      </c>
+      <c r="AN153" s="1">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="154" spans="1:40" x14ac:dyDescent="0.25">
+      <c r="A154" s="10">
+        <v>45900</v>
+      </c>
+      <c r="B154" s="1">
+        <v>84.5</v>
+      </c>
+      <c r="C154" s="1">
+        <v>52.5</v>
+      </c>
+      <c r="D154" s="1">
+        <v>0</v>
+      </c>
+      <c r="E154" s="1">
+        <v>0</v>
+      </c>
+      <c r="F154" s="1">
+        <v>197</v>
+      </c>
+      <c r="G154" s="1">
+        <v>159.5</v>
+      </c>
+      <c r="H154" s="1">
+        <v>8.5</v>
+      </c>
+      <c r="I154" s="1">
+        <v>0</v>
+      </c>
+      <c r="J154" s="1"/>
+      <c r="K154" s="1">
+        <v>0</v>
+      </c>
+      <c r="L154" s="1">
+        <v>560</v>
+      </c>
+      <c r="M154" s="1">
+        <v>0</v>
+      </c>
+      <c r="N154" s="1">
+        <v>0</v>
+      </c>
+      <c r="O154" s="1">
+        <v>11</v>
+      </c>
+      <c r="P154" s="1">
+        <v>0</v>
+      </c>
+      <c r="Q154" s="1">
+        <v>0</v>
+      </c>
+      <c r="R154" s="1">
+        <v>63</v>
+      </c>
+      <c r="S154" s="1">
+        <v>21.5</v>
+      </c>
+      <c r="T154" s="1">
+        <v>0</v>
+      </c>
+      <c r="U154" s="1">
+        <v>51.5</v>
+      </c>
+      <c r="V154" s="1">
+        <v>1</v>
+      </c>
+      <c r="W154" s="1">
+        <v>0</v>
+      </c>
+      <c r="X154" s="1">
+        <v>0</v>
+      </c>
+      <c r="Y154" s="1">
+        <v>0</v>
+      </c>
+      <c r="Z154" s="1">
+        <v>0</v>
+      </c>
+      <c r="AA154" s="1">
+        <v>0</v>
+      </c>
+      <c r="AB154" s="1">
+        <v>0</v>
+      </c>
+      <c r="AC154" s="1">
+        <v>0</v>
+      </c>
+      <c r="AD154" s="1">
+        <v>172.5</v>
+      </c>
+      <c r="AE154" s="1">
+        <v>24.5</v>
+      </c>
+      <c r="AF154" s="1">
+        <v>0</v>
+      </c>
+      <c r="AG154" s="1">
+        <v>28</v>
+      </c>
+      <c r="AH154" s="1">
+        <v>131.5</v>
+      </c>
+      <c r="AI154" s="1">
+        <v>0</v>
+      </c>
+      <c r="AJ154" s="1">
+        <v>7.5</v>
+      </c>
+      <c r="AK154" s="1">
+        <v>1</v>
+      </c>
+      <c r="AL154" s="1">
+        <v>0</v>
+      </c>
+      <c r="AM154" s="1">
+        <v>0</v>
+      </c>
+      <c r="AN154" s="1">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="155" spans="1:40" x14ac:dyDescent="0.25">
+      <c r="A155" s="10">
+        <v>45901</v>
+      </c>
+      <c r="B155" s="1">
+        <v>176</v>
+      </c>
+      <c r="C155" s="1">
+        <v>89</v>
+      </c>
+      <c r="D155" s="1">
+        <v>0</v>
+      </c>
+      <c r="E155" s="1">
+        <v>0</v>
+      </c>
+      <c r="F155" s="1">
+        <v>295</v>
+      </c>
+      <c r="G155" s="1">
+        <v>232</v>
+      </c>
+      <c r="H155" s="1">
+        <v>7</v>
+      </c>
+      <c r="I155" s="1">
+        <v>0</v>
+      </c>
+      <c r="J155" s="1"/>
+      <c r="K155" s="1">
+        <v>0</v>
+      </c>
+      <c r="L155" s="1">
+        <v>768</v>
+      </c>
+      <c r="M155" s="1">
+        <v>0</v>
+      </c>
+      <c r="N155" s="1">
+        <v>0</v>
+      </c>
+      <c r="O155" s="1">
+        <v>0</v>
+      </c>
+      <c r="P155" s="1">
+        <v>0</v>
+      </c>
+      <c r="Q155" s="1">
+        <v>0</v>
+      </c>
+      <c r="R155" s="1">
+        <v>141</v>
+      </c>
+      <c r="S155" s="1">
+        <v>35</v>
+      </c>
+      <c r="T155" s="1">
+        <v>0</v>
+      </c>
+      <c r="U155" s="1">
+        <v>82</v>
+      </c>
+      <c r="V155" s="1">
+        <v>7</v>
+      </c>
+      <c r="W155" s="1">
+        <v>0</v>
+      </c>
+      <c r="X155" s="1">
+        <v>0</v>
+      </c>
+      <c r="Y155" s="1">
+        <v>0</v>
+      </c>
+      <c r="Z155" s="1">
+        <v>0</v>
+      </c>
+      <c r="AA155" s="1">
+        <v>0</v>
+      </c>
+      <c r="AB155" s="1">
+        <v>0</v>
+      </c>
+      <c r="AC155" s="1">
+        <v>0</v>
+      </c>
+      <c r="AD155" s="1">
+        <v>273</v>
+      </c>
+      <c r="AE155" s="1">
+        <v>22</v>
+      </c>
+      <c r="AF155" s="1">
+        <v>0</v>
+      </c>
+      <c r="AG155" s="1">
+        <v>44</v>
+      </c>
+      <c r="AH155" s="1">
+        <v>188</v>
+      </c>
+      <c r="AI155" s="1">
+        <v>0</v>
+      </c>
+      <c r="AJ155" s="1">
+        <v>2</v>
+      </c>
+      <c r="AK155" s="1">
+        <v>5</v>
+      </c>
+      <c r="AL155" s="1">
+        <v>0</v>
+      </c>
+      <c r="AM155" s="1">
+        <v>0</v>
+      </c>
+      <c r="AN155" s="1">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="156" spans="1:40" x14ac:dyDescent="0.25">
+      <c r="A156" s="10">
+        <v>45902</v>
+      </c>
+      <c r="B156" s="1">
+        <v>106</v>
+      </c>
+      <c r="C156" s="1">
+        <v>32</v>
+      </c>
+      <c r="D156" s="1">
+        <v>0</v>
+      </c>
+      <c r="E156" s="1">
+        <v>0</v>
+      </c>
+      <c r="F156" s="1">
+        <v>115</v>
+      </c>
+      <c r="G156" s="1">
+        <v>57</v>
+      </c>
+      <c r="H156" s="1">
+        <v>0</v>
+      </c>
+      <c r="I156" s="1">
+        <v>0</v>
+      </c>
+      <c r="J156" s="1"/>
+      <c r="K156" s="1">
+        <v>0</v>
+      </c>
+      <c r="L156" s="1">
+        <v>254</v>
+      </c>
+      <c r="M156" s="1">
+        <v>0</v>
+      </c>
+      <c r="N156" s="1">
+        <v>0</v>
+      </c>
+      <c r="O156" s="1">
+        <v>18</v>
+      </c>
+      <c r="P156" s="1">
+        <v>0</v>
+      </c>
+      <c r="Q156" s="1">
+        <v>0</v>
+      </c>
+      <c r="R156" s="1">
+        <v>88</v>
+      </c>
+      <c r="S156" s="1">
+        <v>18</v>
+      </c>
+      <c r="T156" s="1">
+        <v>0</v>
+      </c>
+      <c r="U156" s="1">
+        <v>29</v>
+      </c>
+      <c r="V156" s="1">
+        <v>3</v>
+      </c>
+      <c r="W156" s="1">
+        <v>0</v>
+      </c>
+      <c r="X156" s="1">
+        <v>0</v>
+      </c>
+      <c r="Y156" s="1">
+        <v>0</v>
+      </c>
+      <c r="Z156" s="1">
+        <v>0</v>
+      </c>
+      <c r="AA156" s="1">
+        <v>0</v>
+      </c>
+      <c r="AB156" s="1">
+        <v>0</v>
+      </c>
+      <c r="AC156" s="1">
+        <v>0</v>
+      </c>
+      <c r="AD156" s="1">
+        <v>99</v>
+      </c>
+      <c r="AE156" s="1">
         <v>16</v>
       </c>
-      <c r="W150" s="1">
-        <v>0</v>
-      </c>
-      <c r="X150" s="1">
-        <v>0</v>
-      </c>
-      <c r="Y150" s="1">
-        <v>0</v>
-      </c>
-      <c r="Z150" s="1">
-        <v>0</v>
-      </c>
-      <c r="AA150" s="1">
-        <v>0</v>
-      </c>
-      <c r="AB150" s="1">
-        <v>0</v>
-      </c>
-      <c r="AC150" s="1">
-        <v>0</v>
-      </c>
-      <c r="AD150" s="1">
-        <v>3477.5</v>
-      </c>
-      <c r="AE150" s="1">
-        <v>419</v>
-      </c>
-      <c r="AF150" s="1">
-        <v>0</v>
-      </c>
-      <c r="AG150" s="1">
-        <v>129.5</v>
-      </c>
-      <c r="AH150" s="1">
-        <v>560.5</v>
-      </c>
-      <c r="AI150" s="1">
-        <v>0</v>
-      </c>
-      <c r="AJ150" s="1">
-        <v>767</v>
-      </c>
-      <c r="AK150" s="1">
-        <v>102</v>
-      </c>
-      <c r="AL150" s="1">
-        <v>0</v>
-      </c>
-      <c r="AM150" s="1">
-        <v>15</v>
-      </c>
-      <c r="AN150" s="1">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="151" spans="1:40" x14ac:dyDescent="0.25">
-      <c r="A151" s="10"/>
-      <c r="B151" s="1"/>
-      <c r="C151" s="1"/>
-      <c r="D151" s="1"/>
-      <c r="E151" s="1"/>
-      <c r="F151" s="1"/>
-      <c r="G151" s="1"/>
-      <c r="H151" s="1"/>
-      <c r="I151" s="1"/>
-    </row>
-    <row r="152" spans="1:40" x14ac:dyDescent="0.25">
-      <c r="A152" s="10"/>
-      <c r="B152" s="1"/>
-      <c r="C152" s="1"/>
-      <c r="D152" s="1"/>
-      <c r="E152" s="1"/>
-      <c r="F152" s="1"/>
-      <c r="G152" s="1"/>
-      <c r="H152" s="1"/>
-      <c r="I152" s="1"/>
-    </row>
-    <row r="153" spans="1:40" x14ac:dyDescent="0.25">
-      <c r="A153" s="10"/>
-      <c r="B153" s="1"/>
-      <c r="C153" s="1"/>
-      <c r="D153" s="1"/>
-      <c r="E153" s="1"/>
-      <c r="F153" s="1"/>
-      <c r="G153" s="1"/>
-      <c r="H153" s="1"/>
-      <c r="I153" s="1"/>
-    </row>
-    <row r="154" spans="1:40" x14ac:dyDescent="0.25">
-      <c r="A154" s="10"/>
-      <c r="B154" s="1"/>
-      <c r="C154" s="1"/>
-      <c r="D154" s="1"/>
-      <c r="E154" s="1"/>
-      <c r="F154" s="1"/>
-      <c r="G154" s="1"/>
-      <c r="H154" s="1"/>
-      <c r="I154" s="1"/>
-    </row>
-    <row r="155" spans="1:40" x14ac:dyDescent="0.25">
-      <c r="A155" s="10"/>
-      <c r="B155" s="1"/>
-      <c r="C155" s="1"/>
-      <c r="D155" s="1"/>
-      <c r="E155" s="1"/>
-      <c r="F155" s="1"/>
-      <c r="G155" s="1"/>
-      <c r="H155" s="1"/>
-      <c r="I155" s="1"/>
-    </row>
-    <row r="156" spans="1:40" x14ac:dyDescent="0.25">
-      <c r="A156" s="10"/>
-      <c r="B156" s="1"/>
-      <c r="C156" s="1"/>
-      <c r="D156" s="1"/>
-      <c r="E156" s="1"/>
-      <c r="F156" s="1"/>
-      <c r="G156" s="1"/>
-      <c r="H156" s="1"/>
-      <c r="I156" s="1"/>
+      <c r="AF156" s="1">
+        <v>0</v>
+      </c>
+      <c r="AG156" s="1">
+        <v>11</v>
+      </c>
+      <c r="AH156" s="1">
+        <v>46</v>
+      </c>
+      <c r="AI156" s="1">
+        <v>0</v>
+      </c>
+      <c r="AJ156" s="1">
+        <v>0</v>
+      </c>
+      <c r="AK156" s="1">
+        <v>0</v>
+      </c>
+      <c r="AL156" s="1">
+        <v>0</v>
+      </c>
+      <c r="AM156" s="1">
+        <v>0</v>
+      </c>
+      <c r="AN156" s="1">
+        <v>0</v>
+      </c>
     </row>
     <row r="157" spans="1:40" x14ac:dyDescent="0.25">
       <c r="A157" s="10"/>
-      <c r="B157" s="1"/>
-      <c r="C157" s="1"/>
-      <c r="D157" s="1"/>
-      <c r="E157" s="1"/>
-      <c r="F157" s="1"/>
-      <c r="G157" s="1"/>
-      <c r="H157" s="1"/>
-      <c r="I157" s="1"/>
+      <c r="B157" s="14">
+        <v>1939.5</v>
+      </c>
+      <c r="C157" s="14">
+        <v>591.5</v>
+      </c>
+      <c r="D157" s="14">
+        <v>0</v>
+      </c>
+      <c r="E157" s="14">
+        <v>0</v>
+      </c>
+      <c r="F157" s="14">
+        <v>5146</v>
+      </c>
+      <c r="G157" s="14">
+        <v>1664.5</v>
+      </c>
+      <c r="H157" s="14">
+        <v>945</v>
+      </c>
+      <c r="I157" s="14">
+        <v>16</v>
+      </c>
+      <c r="J157" s="1"/>
+      <c r="K157" s="1">
+        <v>0</v>
+      </c>
+      <c r="L157" s="1">
+        <v>433900.96</v>
+      </c>
+      <c r="M157" s="1">
+        <v>0</v>
+      </c>
+      <c r="N157" s="1">
+        <v>0</v>
+      </c>
+      <c r="O157" s="1">
+        <v>3759</v>
+      </c>
+      <c r="P157" s="1">
+        <v>0</v>
+      </c>
+      <c r="Q157" s="1">
+        <v>0</v>
+      </c>
+      <c r="R157" s="1">
+        <v>1579</v>
+      </c>
+      <c r="S157" s="1">
+        <v>360.5</v>
+      </c>
+      <c r="T157" s="1">
+        <v>0</v>
+      </c>
+      <c r="U157" s="1">
+        <v>551.5</v>
+      </c>
+      <c r="V157" s="1">
+        <v>40</v>
+      </c>
+      <c r="W157" s="1">
+        <v>0</v>
+      </c>
+      <c r="X157" s="1">
+        <v>0</v>
+      </c>
+      <c r="Y157" s="1">
+        <v>0</v>
+      </c>
+      <c r="Z157" s="1">
+        <v>0</v>
+      </c>
+      <c r="AA157" s="1">
+        <v>0</v>
+      </c>
+      <c r="AB157" s="1">
+        <v>0</v>
+      </c>
+      <c r="AC157" s="1">
+        <v>0</v>
+      </c>
+      <c r="AD157" s="1">
+        <v>4616.5</v>
+      </c>
+      <c r="AE157" s="1">
+        <v>529.5</v>
+      </c>
+      <c r="AF157" s="1">
+        <v>0</v>
+      </c>
+      <c r="AG157" s="1">
+        <v>302</v>
+      </c>
+      <c r="AH157" s="1">
+        <v>1362.5</v>
+      </c>
+      <c r="AI157" s="1">
+        <v>0</v>
+      </c>
+      <c r="AJ157" s="1">
+        <v>826</v>
+      </c>
+      <c r="AK157" s="1">
+        <v>119</v>
+      </c>
+      <c r="AL157" s="1">
+        <v>0</v>
+      </c>
+      <c r="AM157" s="1">
+        <v>15</v>
+      </c>
+      <c r="AN157" s="1">
+        <v>1</v>
+      </c>
     </row>
     <row r="158" spans="1:40" x14ac:dyDescent="0.25">
       <c r="A158" s="10"/>

</xml_diff>

<commit_message>
minor changes to the code
</commit_message>
<xml_diff>
--- a/End-of-season Historic escapement files/Daily Totals by Age 2025.xlsx
+++ b/End-of-season Historic escapement files/Daily Totals by Age 2025.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29029"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29127"/>
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://hupacasath-my.sharepoint.com/personal/graham_hupacasath_ca/Documents/Documents/Graham DOCS/Escapement/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="131" documentId="8_{439EBB09-C0EF-4C9F-A8FE-AAE85C994023}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{687E7163-ED86-41AD-8849-7D36F549A4DB}"/>
+  <xr:revisionPtr revIDLastSave="141" documentId="8_{439EBB09-C0EF-4C9F-A8FE-AAE85C994023}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{67694DB9-83E4-465A-81BB-EEF227C19F45}"/>
   <bookViews>
-    <workbookView xWindow="34680" yWindow="45" windowWidth="15810" windowHeight="15435" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sproat" sheetId="1" r:id="rId1"/>
@@ -8143,35 +8143,37 @@
       <c r="N164" s="1"/>
     </row>
     <row r="165" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A165" s="1"/>
-      <c r="B165" s="17">
-        <v>56829</v>
-      </c>
-      <c r="C165" s="17">
-        <v>46454</v>
-      </c>
-      <c r="D165" s="18">
-        <v>42326.46</v>
-      </c>
-      <c r="E165" s="18">
-        <v>38822.68</v>
-      </c>
-      <c r="F165" s="18">
-        <v>4131.97</v>
-      </c>
-      <c r="G165" s="18">
-        <v>13720.94</v>
-      </c>
-      <c r="H165" s="18">
-        <v>3218.35</v>
-      </c>
-      <c r="I165" s="14">
-        <v>0</v>
-      </c>
-      <c r="J165" s="18">
-        <v>1062.5899999999999</v>
-      </c>
-      <c r="K165" s="14">
+      <c r="A165" s="10">
+        <v>45903</v>
+      </c>
+      <c r="B165" s="1">
+        <v>19</v>
+      </c>
+      <c r="C165" s="1">
+        <v>14</v>
+      </c>
+      <c r="D165" s="1">
+        <v>12.75</v>
+      </c>
+      <c r="E165" s="1">
+        <v>12</v>
+      </c>
+      <c r="F165" s="1">
+        <v>1.5</v>
+      </c>
+      <c r="G165" s="1">
+        <v>5.25</v>
+      </c>
+      <c r="H165" s="1">
+        <v>0.75</v>
+      </c>
+      <c r="I165" s="1">
+        <v>0</v>
+      </c>
+      <c r="J165" s="1">
+        <v>0.75</v>
+      </c>
+      <c r="K165" s="1">
         <v>0</v>
       </c>
       <c r="L165" s="1"/>
@@ -8179,113 +8181,265 @@
       <c r="N165" s="1"/>
     </row>
     <row r="166" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A166" s="10"/>
-      <c r="B166" s="1"/>
-      <c r="C166" s="1"/>
-      <c r="D166" s="1"/>
-      <c r="E166" s="1"/>
-      <c r="F166" s="1"/>
-      <c r="G166" s="1"/>
-      <c r="H166" s="1"/>
-      <c r="I166" s="1"/>
-      <c r="J166" s="1"/>
-      <c r="K166" s="1"/>
+      <c r="A166" s="10">
+        <v>45904</v>
+      </c>
+      <c r="B166" s="1">
+        <v>49</v>
+      </c>
+      <c r="C166" s="1">
+        <v>38</v>
+      </c>
+      <c r="D166" s="1">
+        <v>33.619999999999997</v>
+      </c>
+      <c r="E166" s="1">
+        <v>31.63</v>
+      </c>
+      <c r="F166" s="1">
+        <v>3.96</v>
+      </c>
+      <c r="G166" s="1">
+        <v>13.84</v>
+      </c>
+      <c r="H166" s="1">
+        <v>1.97</v>
+      </c>
+      <c r="I166" s="1">
+        <v>0</v>
+      </c>
+      <c r="J166" s="1">
+        <v>1.97</v>
+      </c>
+      <c r="K166" s="1">
+        <v>0</v>
+      </c>
       <c r="L166" s="1"/>
       <c r="M166" s="1"/>
       <c r="N166" s="1"/>
     </row>
     <row r="167" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A167" s="10"/>
-      <c r="B167" s="1"/>
-      <c r="C167" s="1"/>
-      <c r="D167" s="1"/>
-      <c r="E167" s="1"/>
-      <c r="F167" s="1"/>
-      <c r="G167" s="1"/>
-      <c r="H167" s="1"/>
-      <c r="I167" s="1"/>
-      <c r="J167" s="1"/>
-      <c r="K167" s="1"/>
+      <c r="A167" s="10">
+        <v>45905</v>
+      </c>
+      <c r="B167" s="1">
+        <v>10</v>
+      </c>
+      <c r="C167" s="1">
+        <v>8</v>
+      </c>
+      <c r="D167" s="1">
+        <v>6.96</v>
+      </c>
+      <c r="E167" s="1">
+        <v>6.54</v>
+      </c>
+      <c r="F167" s="1">
+        <v>0.82</v>
+      </c>
+      <c r="G167" s="1">
+        <v>2.86</v>
+      </c>
+      <c r="H167" s="1">
+        <v>0.41</v>
+      </c>
+      <c r="I167" s="1">
+        <v>0</v>
+      </c>
+      <c r="J167" s="1">
+        <v>0.41</v>
+      </c>
+      <c r="K167" s="1">
+        <v>0</v>
+      </c>
       <c r="L167" s="1"/>
       <c r="M167" s="1"/>
       <c r="N167" s="1"/>
     </row>
     <row r="168" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A168" s="10"/>
-      <c r="B168" s="1"/>
-      <c r="C168" s="1"/>
-      <c r="D168" s="1"/>
-      <c r="E168" s="1"/>
-      <c r="F168" s="1"/>
-      <c r="G168" s="1"/>
-      <c r="H168" s="1"/>
-      <c r="I168" s="1"/>
-      <c r="J168" s="1"/>
-      <c r="K168" s="1"/>
+      <c r="A168" s="10">
+        <v>45906</v>
+      </c>
+      <c r="B168" s="1">
+        <v>7</v>
+      </c>
+      <c r="C168" s="1">
+        <v>6</v>
+      </c>
+      <c r="D168" s="1">
+        <v>5.0199999999999996</v>
+      </c>
+      <c r="E168" s="1">
+        <v>4.7300000000000004</v>
+      </c>
+      <c r="F168" s="1">
+        <v>0.59</v>
+      </c>
+      <c r="G168" s="1">
+        <v>2.0699999999999998</v>
+      </c>
+      <c r="H168" s="1">
+        <v>0.3</v>
+      </c>
+      <c r="I168" s="1">
+        <v>0</v>
+      </c>
+      <c r="J168" s="1">
+        <v>0.3</v>
+      </c>
+      <c r="K168" s="1">
+        <v>0</v>
+      </c>
       <c r="L168" s="1"/>
       <c r="M168" s="1"/>
       <c r="N168" s="1"/>
     </row>
     <row r="169" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A169" s="10"/>
-      <c r="B169" s="1"/>
-      <c r="C169" s="1"/>
-      <c r="D169" s="1"/>
-      <c r="E169" s="1"/>
-      <c r="F169" s="1"/>
-      <c r="G169" s="1"/>
-      <c r="H169" s="1"/>
-      <c r="I169" s="1"/>
-      <c r="J169" s="1"/>
-      <c r="K169" s="1"/>
+      <c r="A169" s="10">
+        <v>45907</v>
+      </c>
+      <c r="B169" s="1">
+        <v>12</v>
+      </c>
+      <c r="C169" s="1">
+        <v>10</v>
+      </c>
+      <c r="D169" s="1">
+        <v>8.5</v>
+      </c>
+      <c r="E169" s="1">
+        <v>8</v>
+      </c>
+      <c r="F169" s="1">
+        <v>1</v>
+      </c>
+      <c r="G169" s="1">
+        <v>3.5</v>
+      </c>
+      <c r="H169" s="1">
+        <v>0.5</v>
+      </c>
+      <c r="I169" s="1">
+        <v>0</v>
+      </c>
+      <c r="J169" s="1">
+        <v>0.5</v>
+      </c>
+      <c r="K169" s="1">
+        <v>0</v>
+      </c>
       <c r="L169" s="1"/>
       <c r="M169" s="1"/>
       <c r="N169" s="1"/>
     </row>
     <row r="170" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A170" s="10"/>
-      <c r="B170" s="1"/>
-      <c r="C170" s="1"/>
-      <c r="D170" s="1"/>
-      <c r="E170" s="1"/>
-      <c r="F170" s="1"/>
-      <c r="G170" s="1"/>
-      <c r="H170" s="1"/>
-      <c r="I170" s="1"/>
-      <c r="J170" s="1"/>
-      <c r="K170" s="1"/>
+      <c r="A170" s="10">
+        <v>45908</v>
+      </c>
+      <c r="B170" s="1">
+        <v>5</v>
+      </c>
+      <c r="C170" s="1">
+        <v>4</v>
+      </c>
+      <c r="D170" s="1">
+        <v>3.48</v>
+      </c>
+      <c r="E170" s="1">
+        <v>3.27</v>
+      </c>
+      <c r="F170" s="1">
+        <v>0.41</v>
+      </c>
+      <c r="G170" s="1">
+        <v>1.43</v>
+      </c>
+      <c r="H170" s="1">
+        <v>0.2</v>
+      </c>
+      <c r="I170" s="1">
+        <v>0</v>
+      </c>
+      <c r="J170" s="1">
+        <v>0.2</v>
+      </c>
+      <c r="K170" s="1">
+        <v>0</v>
+      </c>
       <c r="L170" s="1"/>
       <c r="M170" s="1"/>
       <c r="N170" s="1"/>
     </row>
     <row r="171" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A171" s="10"/>
-      <c r="B171" s="1"/>
-      <c r="C171" s="1"/>
-      <c r="D171" s="1"/>
-      <c r="E171" s="1"/>
-      <c r="F171" s="1"/>
-      <c r="G171" s="1"/>
-      <c r="H171" s="1"/>
-      <c r="I171" s="1"/>
-      <c r="J171" s="1"/>
-      <c r="K171" s="1"/>
+      <c r="A171" s="10">
+        <v>45909</v>
+      </c>
+      <c r="B171" s="1">
+        <v>97</v>
+      </c>
+      <c r="C171" s="1">
+        <v>74</v>
+      </c>
+      <c r="D171" s="1">
+        <v>66.069999999999993</v>
+      </c>
+      <c r="E171" s="1">
+        <v>62.18</v>
+      </c>
+      <c r="F171" s="1">
+        <v>7.78</v>
+      </c>
+      <c r="G171" s="1">
+        <v>27.21</v>
+      </c>
+      <c r="H171" s="1">
+        <v>3.88</v>
+      </c>
+      <c r="I171" s="1">
+        <v>0</v>
+      </c>
+      <c r="J171" s="1">
+        <v>3.88</v>
+      </c>
+      <c r="K171" s="1">
+        <v>0</v>
+      </c>
       <c r="L171" s="1"/>
       <c r="M171" s="1"/>
       <c r="N171" s="1"/>
     </row>
     <row r="172" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A172" s="10"/>
-      <c r="B172" s="1"/>
-      <c r="C172" s="1"/>
-      <c r="D172" s="1"/>
-      <c r="E172" s="1"/>
-      <c r="F172" s="1"/>
-      <c r="G172" s="1"/>
-      <c r="H172" s="1"/>
-      <c r="I172" s="1"/>
-      <c r="J172" s="1"/>
-      <c r="K172" s="1"/>
+      <c r="A172" s="1"/>
+      <c r="B172" s="17">
+        <v>57028</v>
+      </c>
+      <c r="C172" s="17">
+        <v>46608</v>
+      </c>
+      <c r="D172" s="18">
+        <v>42462.86</v>
+      </c>
+      <c r="E172" s="18">
+        <v>38951.03</v>
+      </c>
+      <c r="F172" s="18">
+        <v>4148.03</v>
+      </c>
+      <c r="G172" s="18">
+        <v>13777.11</v>
+      </c>
+      <c r="H172" s="18">
+        <v>3226.37</v>
+      </c>
+      <c r="I172" s="14">
+        <v>0</v>
+      </c>
+      <c r="J172" s="18">
+        <v>1070.5999999999999</v>
+      </c>
+      <c r="K172" s="14">
+        <v>0</v>
+      </c>
       <c r="L172" s="1"/>
       <c r="M172" s="1"/>
       <c r="N172" s="1"/>
@@ -14195,25 +14349,25 @@
         <v>45865</v>
       </c>
       <c r="B120" s="15">
-        <v>5400</v>
+        <v>5478</v>
       </c>
       <c r="C120" s="15">
-        <v>2283</v>
+        <v>2316</v>
       </c>
       <c r="D120" s="16">
-        <v>1836.24</v>
+        <v>1863.01</v>
       </c>
       <c r="E120" s="16">
-        <v>3190.75</v>
+        <v>3236.26</v>
       </c>
       <c r="F120" s="1">
-        <v>446.38</v>
+        <v>452.89</v>
       </c>
       <c r="G120" s="16">
-        <v>1031.83</v>
+        <v>1046.8699999999999</v>
       </c>
       <c r="H120" s="16">
-        <v>1177.8</v>
+        <v>1194.97</v>
       </c>
       <c r="I120" s="1">
         <v>0</v>
@@ -15527,31 +15681,31 @@
         <v>45902</v>
       </c>
       <c r="B157" s="1">
-        <v>191</v>
+        <v>443</v>
       </c>
       <c r="C157" s="1">
-        <v>81</v>
+        <v>188</v>
       </c>
       <c r="D157" s="1">
-        <v>75.239999999999995</v>
+        <v>174.53</v>
       </c>
       <c r="E157" s="1">
-        <v>109.94</v>
+        <v>255.05</v>
       </c>
       <c r="F157" s="1">
-        <v>5.79</v>
+        <v>13.44</v>
       </c>
       <c r="G157" s="1">
-        <v>28.94</v>
+        <v>67.14</v>
       </c>
       <c r="H157" s="1">
-        <v>46.29</v>
+        <v>107.4</v>
       </c>
       <c r="I157" s="1">
         <v>0</v>
       </c>
       <c r="J157" s="1">
-        <v>5.79</v>
+        <v>13.44</v>
       </c>
       <c r="K157" s="1">
         <v>0</v>
@@ -15559,135 +15713,289 @@
       <c r="L157" s="1"/>
     </row>
     <row r="158" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A158" s="1"/>
-      <c r="B158" s="17">
-        <v>332959</v>
-      </c>
-      <c r="C158" s="17">
-        <v>104705</v>
-      </c>
-      <c r="D158" s="18">
-        <v>90164.82</v>
-      </c>
-      <c r="E158" s="18">
-        <v>200149</v>
-      </c>
-      <c r="F158" s="18">
-        <v>14544.8</v>
-      </c>
-      <c r="G158" s="18">
-        <v>65376.68</v>
-      </c>
-      <c r="H158" s="18">
-        <v>63897.04</v>
-      </c>
-      <c r="I158" s="14">
-        <v>0</v>
-      </c>
-      <c r="J158" s="18">
-        <v>3531.68</v>
-      </c>
-      <c r="K158" s="14">
+      <c r="A158" s="10">
+        <v>45903</v>
+      </c>
+      <c r="B158" s="1">
+        <v>397</v>
+      </c>
+      <c r="C158" s="1">
+        <v>168</v>
+      </c>
+      <c r="D158" s="1">
+        <v>156.28</v>
+      </c>
+      <c r="E158" s="1">
+        <v>228.37</v>
+      </c>
+      <c r="F158" s="1">
+        <v>12.03</v>
+      </c>
+      <c r="G158" s="1">
+        <v>60.12</v>
+      </c>
+      <c r="H158" s="1">
+        <v>96.16</v>
+      </c>
+      <c r="I158" s="1">
+        <v>0</v>
+      </c>
+      <c r="J158" s="1">
+        <v>12.03</v>
+      </c>
+      <c r="K158" s="1">
         <v>0</v>
       </c>
       <c r="L158" s="1"/>
     </row>
     <row r="159" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A159" s="10"/>
-      <c r="B159" s="1"/>
-      <c r="C159" s="1"/>
-      <c r="D159" s="1"/>
-      <c r="E159" s="1"/>
-      <c r="F159" s="1"/>
-      <c r="G159" s="1"/>
-      <c r="H159" s="1"/>
-      <c r="I159" s="1"/>
-      <c r="J159" s="1"/>
-      <c r="K159" s="1"/>
+      <c r="A159" s="10">
+        <v>45904</v>
+      </c>
+      <c r="B159" s="1">
+        <v>393</v>
+      </c>
+      <c r="C159" s="1">
+        <v>167</v>
+      </c>
+      <c r="D159" s="1">
+        <v>154.9</v>
+      </c>
+      <c r="E159" s="1">
+        <v>226.35</v>
+      </c>
+      <c r="F159" s="1">
+        <v>11.93</v>
+      </c>
+      <c r="G159" s="1">
+        <v>59.58</v>
+      </c>
+      <c r="H159" s="1">
+        <v>95.31</v>
+      </c>
+      <c r="I159" s="1">
+        <v>0</v>
+      </c>
+      <c r="J159" s="1">
+        <v>11.93</v>
+      </c>
+      <c r="K159" s="1">
+        <v>0</v>
+      </c>
       <c r="L159" s="1"/>
     </row>
     <row r="160" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A160" s="10"/>
-      <c r="B160" s="1"/>
-      <c r="C160" s="1"/>
-      <c r="D160" s="1"/>
-      <c r="E160" s="1"/>
-      <c r="F160" s="1"/>
-      <c r="G160" s="1"/>
-      <c r="H160" s="1"/>
-      <c r="I160" s="1"/>
-      <c r="J160" s="1"/>
-      <c r="K160" s="1"/>
+      <c r="A160" s="10">
+        <v>45905</v>
+      </c>
+      <c r="B160" s="1">
+        <v>209</v>
+      </c>
+      <c r="C160" s="1">
+        <v>89</v>
+      </c>
+      <c r="D160" s="1">
+        <v>82.43</v>
+      </c>
+      <c r="E160" s="1">
+        <v>120.45</v>
+      </c>
+      <c r="F160" s="1">
+        <v>6.35</v>
+      </c>
+      <c r="G160" s="1">
+        <v>31.71</v>
+      </c>
+      <c r="H160" s="1">
+        <v>50.72</v>
+      </c>
+      <c r="I160" s="1">
+        <v>0</v>
+      </c>
+      <c r="J160" s="1">
+        <v>6.35</v>
+      </c>
+      <c r="K160" s="1">
+        <v>0</v>
+      </c>
       <c r="L160" s="1"/>
     </row>
     <row r="161" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A161" s="10"/>
-      <c r="B161" s="1"/>
-      <c r="C161" s="1"/>
-      <c r="D161" s="1"/>
-      <c r="E161" s="1"/>
-      <c r="F161" s="1"/>
-      <c r="G161" s="1"/>
-      <c r="H161" s="1"/>
-      <c r="I161" s="1"/>
-      <c r="J161" s="1"/>
-      <c r="K161" s="1"/>
+      <c r="A161" s="10">
+        <v>45906</v>
+      </c>
+      <c r="B161" s="1">
+        <v>145</v>
+      </c>
+      <c r="C161" s="1">
+        <v>61</v>
+      </c>
+      <c r="D161" s="1">
+        <v>56.98</v>
+      </c>
+      <c r="E161" s="1">
+        <v>83.27</v>
+      </c>
+      <c r="F161" s="1">
+        <v>4.3899999999999997</v>
+      </c>
+      <c r="G161" s="1">
+        <v>21.92</v>
+      </c>
+      <c r="H161" s="1">
+        <v>35.06</v>
+      </c>
+      <c r="I161" s="1">
+        <v>0</v>
+      </c>
+      <c r="J161" s="1">
+        <v>4.3899999999999997</v>
+      </c>
+      <c r="K161" s="1">
+        <v>0</v>
+      </c>
       <c r="L161" s="1"/>
     </row>
     <row r="162" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A162" s="10"/>
-      <c r="B162" s="1"/>
-      <c r="C162" s="1"/>
-      <c r="D162" s="1"/>
-      <c r="E162" s="1"/>
-      <c r="F162" s="1"/>
-      <c r="G162" s="1"/>
-      <c r="H162" s="1"/>
-      <c r="I162" s="1"/>
-      <c r="J162" s="1"/>
-      <c r="K162" s="1"/>
+      <c r="A162" s="10">
+        <v>45907</v>
+      </c>
+      <c r="B162" s="1">
+        <v>206</v>
+      </c>
+      <c r="C162" s="1">
+        <v>88</v>
+      </c>
+      <c r="D162" s="1">
+        <v>81.319999999999993</v>
+      </c>
+      <c r="E162" s="1">
+        <v>118.83</v>
+      </c>
+      <c r="F162" s="1">
+        <v>6.26</v>
+      </c>
+      <c r="G162" s="1">
+        <v>31.28</v>
+      </c>
+      <c r="H162" s="1">
+        <v>50.04</v>
+      </c>
+      <c r="I162" s="1">
+        <v>0</v>
+      </c>
+      <c r="J162" s="1">
+        <v>6.26</v>
+      </c>
+      <c r="K162" s="1">
+        <v>0</v>
+      </c>
       <c r="L162" s="1"/>
     </row>
     <row r="163" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A163" s="10"/>
-      <c r="B163" s="1"/>
-      <c r="C163" s="1"/>
-      <c r="D163" s="1"/>
-      <c r="E163" s="1"/>
-      <c r="F163" s="1"/>
-      <c r="G163" s="1"/>
-      <c r="H163" s="1"/>
-      <c r="I163" s="1"/>
-      <c r="J163" s="1"/>
-      <c r="K163" s="1"/>
+      <c r="A163" s="10">
+        <v>45908</v>
+      </c>
+      <c r="B163" s="1">
+        <v>269</v>
+      </c>
+      <c r="C163" s="1">
+        <v>114</v>
+      </c>
+      <c r="D163" s="1">
+        <v>105.94</v>
+      </c>
+      <c r="E163" s="1">
+        <v>154.81</v>
+      </c>
+      <c r="F163" s="1">
+        <v>8.16</v>
+      </c>
+      <c r="G163" s="1">
+        <v>40.75</v>
+      </c>
+      <c r="H163" s="1">
+        <v>65.19</v>
+      </c>
+      <c r="I163" s="1">
+        <v>0</v>
+      </c>
+      <c r="J163" s="1">
+        <v>8.16</v>
+      </c>
+      <c r="K163" s="1">
+        <v>0</v>
+      </c>
       <c r="L163" s="1"/>
     </row>
     <row r="164" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A164" s="10"/>
-      <c r="B164" s="1"/>
-      <c r="C164" s="1"/>
-      <c r="D164" s="1"/>
-      <c r="E164" s="1"/>
-      <c r="F164" s="1"/>
-      <c r="G164" s="1"/>
-      <c r="H164" s="1"/>
-      <c r="I164" s="1"/>
-      <c r="J164" s="1"/>
-      <c r="K164" s="1"/>
+      <c r="A164" s="10">
+        <v>45909</v>
+      </c>
+      <c r="B164" s="1">
+        <v>415</v>
+      </c>
+      <c r="C164" s="1">
+        <v>176</v>
+      </c>
+      <c r="D164" s="1">
+        <v>163.47</v>
+      </c>
+      <c r="E164" s="1">
+        <v>238.88</v>
+      </c>
+      <c r="F164" s="1">
+        <v>12.59</v>
+      </c>
+      <c r="G164" s="1">
+        <v>62.88</v>
+      </c>
+      <c r="H164" s="1">
+        <v>100.59</v>
+      </c>
+      <c r="I164" s="1">
+        <v>0</v>
+      </c>
+      <c r="J164" s="1">
+        <v>12.59</v>
+      </c>
+      <c r="K164" s="1">
+        <v>0</v>
+      </c>
       <c r="L164" s="1"/>
     </row>
     <row r="165" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A165" s="10"/>
-      <c r="B165" s="1"/>
-      <c r="C165" s="1"/>
-      <c r="D165" s="1"/>
-      <c r="E165" s="1"/>
-      <c r="F165" s="1"/>
-      <c r="G165" s="1"/>
-      <c r="H165" s="1"/>
-      <c r="I165" s="1"/>
-      <c r="J165" s="1"/>
-      <c r="K165" s="1"/>
+      <c r="A165" s="1"/>
+      <c r="B165" s="17">
+        <v>335323</v>
+      </c>
+      <c r="C165" s="17">
+        <v>105708</v>
+      </c>
+      <c r="D165" s="18">
+        <v>91092.2</v>
+      </c>
+      <c r="E165" s="18">
+        <v>201510.58</v>
+      </c>
+      <c r="F165" s="18">
+        <v>14620.66</v>
+      </c>
+      <c r="G165" s="18">
+        <v>65738.16</v>
+      </c>
+      <c r="H165" s="18">
+        <v>64468.38</v>
+      </c>
+      <c r="I165" s="14">
+        <v>0</v>
+      </c>
+      <c r="J165" s="18">
+        <v>3601.03</v>
+      </c>
+      <c r="K165" s="14">
+        <v>0</v>
+      </c>
       <c r="L165" s="1"/>
     </row>
     <row r="166" spans="1:12" x14ac:dyDescent="0.25">
@@ -21219,108 +21527,234 @@
       </c>
     </row>
     <row r="164" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A164" s="10"/>
-      <c r="B164" s="14">
-        <v>4452.76</v>
-      </c>
-      <c r="C164" s="14">
-        <v>388.99</v>
-      </c>
-      <c r="D164" s="14">
-        <v>1.22</v>
-      </c>
-      <c r="E164" s="14">
-        <v>0</v>
-      </c>
-      <c r="F164" s="14">
-        <v>1.0900000000000001</v>
-      </c>
-      <c r="G164" s="14">
-        <v>1.33</v>
-      </c>
-      <c r="H164" s="14">
-        <v>65.72</v>
-      </c>
-      <c r="I164" s="14">
-        <v>11.36</v>
+      <c r="A164" s="10">
+        <v>45903</v>
+      </c>
+      <c r="B164" s="1">
+        <v>141.24</v>
+      </c>
+      <c r="C164" s="1">
+        <v>61.51</v>
+      </c>
+      <c r="D164" s="1">
+        <v>0</v>
+      </c>
+      <c r="E164" s="1">
+        <v>0</v>
+      </c>
+      <c r="F164" s="1">
+        <v>0</v>
+      </c>
+      <c r="G164" s="1">
+        <v>0</v>
+      </c>
+      <c r="H164" s="1">
+        <v>0</v>
+      </c>
+      <c r="I164" s="1">
+        <v>0</v>
       </c>
     </row>
     <row r="165" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A165" s="10"/>
-      <c r="B165" s="1"/>
-      <c r="C165" s="1"/>
-      <c r="D165" s="1"/>
-      <c r="E165" s="1"/>
-      <c r="F165" s="1"/>
-      <c r="G165" s="1"/>
-      <c r="H165" s="1"/>
-      <c r="I165" s="1"/>
+      <c r="A165" s="10">
+        <v>45904</v>
+      </c>
+      <c r="B165" s="1">
+        <v>100.53</v>
+      </c>
+      <c r="C165" s="1">
+        <v>1.17</v>
+      </c>
+      <c r="D165" s="1">
+        <v>0</v>
+      </c>
+      <c r="E165" s="1">
+        <v>0</v>
+      </c>
+      <c r="F165" s="1">
+        <v>0</v>
+      </c>
+      <c r="G165" s="1">
+        <v>0</v>
+      </c>
+      <c r="H165" s="1">
+        <v>0</v>
+      </c>
+      <c r="I165" s="1">
+        <v>0</v>
+      </c>
     </row>
     <row r="166" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A166" s="10"/>
-      <c r="B166" s="1"/>
-      <c r="C166" s="1"/>
-      <c r="D166" s="1"/>
-      <c r="E166" s="1"/>
-      <c r="F166" s="1"/>
-      <c r="G166" s="1"/>
-      <c r="H166" s="1"/>
-      <c r="I166" s="1"/>
+      <c r="A166" s="10">
+        <v>45905</v>
+      </c>
+      <c r="B166" s="1">
+        <v>147.47999999999999</v>
+      </c>
+      <c r="C166" s="1">
+        <v>55.15</v>
+      </c>
+      <c r="D166" s="1">
+        <v>0</v>
+      </c>
+      <c r="E166" s="1">
+        <v>0</v>
+      </c>
+      <c r="F166" s="1">
+        <v>0</v>
+      </c>
+      <c r="G166" s="1">
+        <v>0</v>
+      </c>
+      <c r="H166" s="1">
+        <v>0</v>
+      </c>
+      <c r="I166" s="1">
+        <v>0</v>
+      </c>
     </row>
     <row r="167" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A167" s="10"/>
-      <c r="B167" s="1"/>
-      <c r="C167" s="1"/>
-      <c r="D167" s="1"/>
-      <c r="E167" s="1"/>
-      <c r="F167" s="1"/>
-      <c r="G167" s="1"/>
-      <c r="H167" s="1"/>
-      <c r="I167" s="1"/>
+      <c r="A167" s="10">
+        <v>45906</v>
+      </c>
+      <c r="B167" s="1">
+        <v>132.84</v>
+      </c>
+      <c r="C167" s="1">
+        <v>57.81</v>
+      </c>
+      <c r="D167" s="1">
+        <v>0</v>
+      </c>
+      <c r="E167" s="1">
+        <v>0</v>
+      </c>
+      <c r="F167" s="1">
+        <v>0</v>
+      </c>
+      <c r="G167" s="1">
+        <v>0</v>
+      </c>
+      <c r="H167" s="1">
+        <v>0</v>
+      </c>
+      <c r="I167" s="1">
+        <v>0</v>
+      </c>
     </row>
     <row r="168" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A168" s="10"/>
-      <c r="B168" s="1"/>
-      <c r="C168" s="1"/>
-      <c r="D168" s="1"/>
-      <c r="E168" s="1"/>
-      <c r="F168" s="1"/>
-      <c r="G168" s="1"/>
-      <c r="H168" s="1"/>
-      <c r="I168" s="1"/>
+      <c r="A168" s="10">
+        <v>45907</v>
+      </c>
+      <c r="B168" s="1">
+        <v>265.68</v>
+      </c>
+      <c r="C168" s="1">
+        <v>81.180000000000007</v>
+      </c>
+      <c r="D168" s="1">
+        <v>0</v>
+      </c>
+      <c r="E168" s="1">
+        <v>0</v>
+      </c>
+      <c r="F168" s="1">
+        <v>0</v>
+      </c>
+      <c r="G168" s="1">
+        <v>0</v>
+      </c>
+      <c r="H168" s="1">
+        <v>0</v>
+      </c>
+      <c r="I168" s="1">
+        <v>0</v>
+      </c>
     </row>
     <row r="169" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A169" s="10"/>
-      <c r="B169" s="1"/>
-      <c r="C169" s="1"/>
-      <c r="D169" s="1"/>
-      <c r="E169" s="1"/>
-      <c r="F169" s="1"/>
-      <c r="G169" s="1"/>
-      <c r="H169" s="1"/>
-      <c r="I169" s="1"/>
+      <c r="A169" s="10">
+        <v>45908</v>
+      </c>
+      <c r="B169" s="1">
+        <v>307.5</v>
+      </c>
+      <c r="C169" s="1">
+        <v>59.04</v>
+      </c>
+      <c r="D169" s="1">
+        <v>0</v>
+      </c>
+      <c r="E169" s="1">
+        <v>0</v>
+      </c>
+      <c r="F169" s="1">
+        <v>0</v>
+      </c>
+      <c r="G169" s="1">
+        <v>0</v>
+      </c>
+      <c r="H169" s="1">
+        <v>0</v>
+      </c>
+      <c r="I169" s="1">
+        <v>0</v>
+      </c>
     </row>
     <row r="170" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A170" s="10"/>
-      <c r="B170" s="1"/>
-      <c r="C170" s="1"/>
-      <c r="D170" s="1"/>
-      <c r="E170" s="1"/>
-      <c r="F170" s="1"/>
-      <c r="G170" s="1"/>
-      <c r="H170" s="1"/>
-      <c r="I170" s="1"/>
+      <c r="A170" s="10">
+        <v>45909</v>
+      </c>
+      <c r="B170" s="1">
+        <v>296.43</v>
+      </c>
+      <c r="C170" s="1">
+        <v>0</v>
+      </c>
+      <c r="D170" s="1">
+        <v>0</v>
+      </c>
+      <c r="E170" s="1">
+        <v>0</v>
+      </c>
+      <c r="F170" s="1">
+        <v>0</v>
+      </c>
+      <c r="G170" s="1">
+        <v>0</v>
+      </c>
+      <c r="H170" s="1">
+        <v>0</v>
+      </c>
+      <c r="I170" s="1">
+        <v>0</v>
+      </c>
     </row>
     <row r="171" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A171" s="10"/>
-      <c r="B171" s="1"/>
-      <c r="C171" s="1"/>
-      <c r="D171" s="1"/>
-      <c r="E171" s="1"/>
-      <c r="F171" s="1"/>
-      <c r="G171" s="1"/>
-      <c r="H171" s="1"/>
-      <c r="I171" s="1"/>
+      <c r="B171" s="14">
+        <v>5844.46</v>
+      </c>
+      <c r="C171" s="14">
+        <v>704.85</v>
+      </c>
+      <c r="D171" s="14">
+        <v>1.22</v>
+      </c>
+      <c r="E171" s="14">
+        <v>0</v>
+      </c>
+      <c r="F171" s="14">
+        <v>1.0900000000000001</v>
+      </c>
+      <c r="G171" s="14">
+        <v>1.33</v>
+      </c>
+      <c r="H171" s="14">
+        <v>65.72</v>
+      </c>
+      <c r="I171" s="14">
+        <v>11.36</v>
+      </c>
     </row>
     <row r="172" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A172" s="10"/>
@@ -36374,7 +36808,7 @@
         <v>0</v>
       </c>
       <c r="L119" s="1">
-        <v>7683</v>
+        <v>7795</v>
       </c>
       <c r="M119" s="1">
         <v>0</v>
@@ -40786,10 +41220,10 @@
         <v>45902</v>
       </c>
       <c r="B156" s="1">
-        <v>106</v>
+        <v>243</v>
       </c>
       <c r="C156" s="1">
-        <v>32</v>
+        <v>95</v>
       </c>
       <c r="D156" s="1">
         <v>0</v>
@@ -40798,13 +41232,13 @@
         <v>0</v>
       </c>
       <c r="F156" s="1">
-        <v>115</v>
+        <v>510</v>
       </c>
       <c r="G156" s="1">
-        <v>57</v>
+        <v>304</v>
       </c>
       <c r="H156" s="1">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I156" s="1">
         <v>0</v>
@@ -40814,7 +41248,7 @@
         <v>0</v>
       </c>
       <c r="L156" s="1">
-        <v>254</v>
+        <v>585</v>
       </c>
       <c r="M156" s="1">
         <v>0</v>
@@ -40823,7 +41257,7 @@
         <v>0</v>
       </c>
       <c r="O156" s="1">
-        <v>18</v>
+        <v>46</v>
       </c>
       <c r="P156" s="1">
         <v>0</v>
@@ -40832,107 +41266,109 @@
         <v>0</v>
       </c>
       <c r="R156" s="1">
+        <v>179</v>
+      </c>
+      <c r="S156" s="1">
+        <v>64</v>
+      </c>
+      <c r="T156" s="1">
+        <v>0</v>
+      </c>
+      <c r="U156" s="1">
+        <v>85</v>
+      </c>
+      <c r="V156" s="1">
+        <v>10</v>
+      </c>
+      <c r="W156" s="1">
+        <v>0</v>
+      </c>
+      <c r="X156" s="1">
+        <v>0</v>
+      </c>
+      <c r="Y156" s="1">
+        <v>0</v>
+      </c>
+      <c r="Z156" s="1">
+        <v>0</v>
+      </c>
+      <c r="AA156" s="1">
+        <v>0</v>
+      </c>
+      <c r="AB156" s="1">
+        <v>0</v>
+      </c>
+      <c r="AC156" s="1">
+        <v>0</v>
+      </c>
+      <c r="AD156" s="1">
+        <v>451</v>
+      </c>
+      <c r="AE156" s="1">
+        <v>59</v>
+      </c>
+      <c r="AF156" s="1">
+        <v>0</v>
+      </c>
+      <c r="AG156" s="1">
+        <v>55</v>
+      </c>
+      <c r="AH156" s="1">
+        <v>249</v>
+      </c>
+      <c r="AI156" s="1">
+        <v>0</v>
+      </c>
+      <c r="AJ156" s="1">
+        <v>1</v>
+      </c>
+      <c r="AK156" s="1">
+        <v>0</v>
+      </c>
+      <c r="AL156" s="1">
+        <v>0</v>
+      </c>
+      <c r="AM156" s="1">
+        <v>0</v>
+      </c>
+      <c r="AN156" s="1">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="157" spans="1:40" x14ac:dyDescent="0.25">
+      <c r="A157" s="10">
+        <v>45903</v>
+      </c>
+      <c r="B157" s="1">
+        <v>227</v>
+      </c>
+      <c r="C157" s="1">
         <v>88</v>
       </c>
-      <c r="S156" s="1">
-        <v>18</v>
-      </c>
-      <c r="T156" s="1">
-        <v>0</v>
-      </c>
-      <c r="U156" s="1">
-        <v>29</v>
-      </c>
-      <c r="V156" s="1">
-        <v>3</v>
-      </c>
-      <c r="W156" s="1">
-        <v>0</v>
-      </c>
-      <c r="X156" s="1">
-        <v>0</v>
-      </c>
-      <c r="Y156" s="1">
-        <v>0</v>
-      </c>
-      <c r="Z156" s="1">
-        <v>0</v>
-      </c>
-      <c r="AA156" s="1">
-        <v>0</v>
-      </c>
-      <c r="AB156" s="1">
-        <v>0</v>
-      </c>
-      <c r="AC156" s="1">
-        <v>0</v>
-      </c>
-      <c r="AD156" s="1">
-        <v>99</v>
-      </c>
-      <c r="AE156" s="1">
-        <v>16</v>
-      </c>
-      <c r="AF156" s="1">
-        <v>0</v>
-      </c>
-      <c r="AG156" s="1">
-        <v>11</v>
-      </c>
-      <c r="AH156" s="1">
-        <v>46</v>
-      </c>
-      <c r="AI156" s="1">
-        <v>0</v>
-      </c>
-      <c r="AJ156" s="1">
-        <v>0</v>
-      </c>
-      <c r="AK156" s="1">
-        <v>0</v>
-      </c>
-      <c r="AL156" s="1">
-        <v>0</v>
-      </c>
-      <c r="AM156" s="1">
-        <v>0</v>
-      </c>
-      <c r="AN156" s="1">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="157" spans="1:40" x14ac:dyDescent="0.25">
-      <c r="A157" s="10"/>
-      <c r="B157" s="14">
-        <v>1939.5</v>
-      </c>
-      <c r="C157" s="14">
-        <v>591.5</v>
-      </c>
-      <c r="D157" s="14">
-        <v>0</v>
-      </c>
-      <c r="E157" s="14">
-        <v>0</v>
-      </c>
-      <c r="F157" s="14">
-        <v>5146</v>
-      </c>
-      <c r="G157" s="14">
-        <v>1664.5</v>
-      </c>
-      <c r="H157" s="14">
-        <v>945</v>
-      </c>
-      <c r="I157" s="14">
-        <v>16</v>
+      <c r="D157" s="1">
+        <v>0</v>
+      </c>
+      <c r="E157" s="1">
+        <v>0</v>
+      </c>
+      <c r="F157" s="1">
+        <v>418</v>
+      </c>
+      <c r="G157" s="1">
+        <v>278</v>
+      </c>
+      <c r="H157" s="1">
+        <v>6</v>
+      </c>
+      <c r="I157" s="1">
+        <v>0</v>
       </c>
       <c r="J157" s="1"/>
       <c r="K157" s="1">
         <v>0</v>
       </c>
       <c r="L157" s="1">
-        <v>433900.96</v>
+        <v>537</v>
       </c>
       <c r="M157" s="1">
         <v>0</v>
@@ -40941,7 +41377,7 @@
         <v>0</v>
       </c>
       <c r="O157" s="1">
-        <v>3759</v>
+        <v>28</v>
       </c>
       <c r="P157" s="1">
         <v>0</v>
@@ -40950,153 +41386,914 @@
         <v>0</v>
       </c>
       <c r="R157" s="1">
-        <v>1579</v>
+        <v>158</v>
       </c>
       <c r="S157" s="1">
-        <v>360.5</v>
+        <v>69</v>
       </c>
       <c r="T157" s="1">
         <v>0</v>
       </c>
       <c r="U157" s="1">
-        <v>551.5</v>
+        <v>80</v>
       </c>
       <c r="V157" s="1">
+        <v>8</v>
+      </c>
+      <c r="W157" s="1">
+        <v>0</v>
+      </c>
+      <c r="X157" s="1">
+        <v>0</v>
+      </c>
+      <c r="Y157" s="1">
+        <v>0</v>
+      </c>
+      <c r="Z157" s="1">
+        <v>0</v>
+      </c>
+      <c r="AA157" s="1">
+        <v>0</v>
+      </c>
+      <c r="AB157" s="1">
+        <v>0</v>
+      </c>
+      <c r="AC157" s="1">
+        <v>0</v>
+      </c>
+      <c r="AD157" s="1">
+        <v>372</v>
+      </c>
+      <c r="AE157" s="1">
+        <v>46</v>
+      </c>
+      <c r="AF157" s="1">
+        <v>0</v>
+      </c>
+      <c r="AG157" s="1">
         <v>40</v>
       </c>
-      <c r="W157" s="1">
-        <v>0</v>
-      </c>
-      <c r="X157" s="1">
-        <v>0</v>
-      </c>
-      <c r="Y157" s="1">
-        <v>0</v>
-      </c>
-      <c r="Z157" s="1">
-        <v>0</v>
-      </c>
-      <c r="AA157" s="1">
-        <v>0</v>
-      </c>
-      <c r="AB157" s="1">
-        <v>0</v>
-      </c>
-      <c r="AC157" s="1">
-        <v>0</v>
-      </c>
-      <c r="AD157" s="1">
-        <v>4616.5</v>
-      </c>
-      <c r="AE157" s="1">
-        <v>529.5</v>
-      </c>
-      <c r="AF157" s="1">
-        <v>0</v>
-      </c>
-      <c r="AG157" s="1">
-        <v>302</v>
-      </c>
       <c r="AH157" s="1">
-        <v>1362.5</v>
+        <v>238</v>
       </c>
       <c r="AI157" s="1">
         <v>0</v>
       </c>
       <c r="AJ157" s="1">
-        <v>826</v>
+        <v>2</v>
       </c>
       <c r="AK157" s="1">
-        <v>119</v>
+        <v>4</v>
       </c>
       <c r="AL157" s="1">
         <v>0</v>
       </c>
       <c r="AM157" s="1">
+        <v>0</v>
+      </c>
+      <c r="AN157" s="1">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="158" spans="1:40" x14ac:dyDescent="0.25">
+      <c r="A158" s="10">
+        <v>45904</v>
+      </c>
+      <c r="B158" s="1">
+        <v>226</v>
+      </c>
+      <c r="C158" s="1">
+        <v>115</v>
+      </c>
+      <c r="D158" s="1">
+        <v>0</v>
+      </c>
+      <c r="E158" s="1">
+        <v>0</v>
+      </c>
+      <c r="F158" s="1">
+        <v>1205</v>
+      </c>
+      <c r="G158" s="1">
+        <v>426</v>
+      </c>
+      <c r="H158" s="1">
+        <v>10</v>
+      </c>
+      <c r="I158" s="1">
+        <v>0</v>
+      </c>
+      <c r="J158" s="1"/>
+      <c r="K158" s="1">
+        <v>0</v>
+      </c>
+      <c r="L158" s="1">
+        <v>560</v>
+      </c>
+      <c r="M158" s="1">
+        <v>0</v>
+      </c>
+      <c r="N158" s="1">
+        <v>0</v>
+      </c>
+      <c r="O158" s="1">
+        <v>0</v>
+      </c>
+      <c r="P158" s="1">
+        <v>0</v>
+      </c>
+      <c r="Q158" s="1">
+        <v>0</v>
+      </c>
+      <c r="R158" s="1">
+        <v>165</v>
+      </c>
+      <c r="S158" s="1">
+        <v>61</v>
+      </c>
+      <c r="T158" s="1">
+        <v>0</v>
+      </c>
+      <c r="U158" s="1">
+        <v>99</v>
+      </c>
+      <c r="V158" s="1">
+        <v>16</v>
+      </c>
+      <c r="W158" s="1">
+        <v>0</v>
+      </c>
+      <c r="X158" s="1">
+        <v>0</v>
+      </c>
+      <c r="Y158" s="1">
+        <v>0</v>
+      </c>
+      <c r="Z158" s="1">
+        <v>0</v>
+      </c>
+      <c r="AA158" s="1">
+        <v>0</v>
+      </c>
+      <c r="AB158" s="1">
+        <v>0</v>
+      </c>
+      <c r="AC158" s="1">
+        <v>0</v>
+      </c>
+      <c r="AD158" s="1">
+        <v>1111</v>
+      </c>
+      <c r="AE158" s="1">
+        <v>94</v>
+      </c>
+      <c r="AF158" s="1">
+        <v>0</v>
+      </c>
+      <c r="AG158" s="1">
+        <v>50</v>
+      </c>
+      <c r="AH158" s="1">
+        <v>376</v>
+      </c>
+      <c r="AI158" s="1">
+        <v>0</v>
+      </c>
+      <c r="AJ158" s="1">
+        <v>8</v>
+      </c>
+      <c r="AK158" s="1">
+        <v>2</v>
+      </c>
+      <c r="AL158" s="1">
+        <v>0</v>
+      </c>
+      <c r="AM158" s="1">
+        <v>0</v>
+      </c>
+      <c r="AN158" s="1">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="159" spans="1:40" x14ac:dyDescent="0.25">
+      <c r="A159" s="10">
+        <v>45905</v>
+      </c>
+      <c r="B159" s="1">
+        <v>199</v>
+      </c>
+      <c r="C159" s="1">
+        <v>104</v>
+      </c>
+      <c r="D159" s="1">
+        <v>0</v>
+      </c>
+      <c r="E159" s="1">
+        <v>0</v>
+      </c>
+      <c r="F159" s="1">
+        <v>810</v>
+      </c>
+      <c r="G159" s="1">
+        <v>280</v>
+      </c>
+      <c r="H159" s="1">
+        <v>10</v>
+      </c>
+      <c r="I159" s="1">
+        <v>0</v>
+      </c>
+      <c r="J159" s="1"/>
+      <c r="K159" s="1">
+        <v>0</v>
+      </c>
+      <c r="L159" s="1">
+        <v>281</v>
+      </c>
+      <c r="M159" s="1">
+        <v>0</v>
+      </c>
+      <c r="N159" s="1">
+        <v>0</v>
+      </c>
+      <c r="O159" s="1">
+        <v>17</v>
+      </c>
+      <c r="P159" s="1">
+        <v>0</v>
+      </c>
+      <c r="Q159" s="1">
+        <v>0</v>
+      </c>
+      <c r="R159" s="1">
+        <v>155</v>
+      </c>
+      <c r="S159" s="1">
+        <v>44</v>
+      </c>
+      <c r="T159" s="1">
+        <v>0</v>
+      </c>
+      <c r="U159" s="1">
+        <v>86</v>
+      </c>
+      <c r="V159" s="1">
+        <v>18</v>
+      </c>
+      <c r="W159" s="1">
+        <v>0</v>
+      </c>
+      <c r="X159" s="1">
+        <v>0</v>
+      </c>
+      <c r="Y159" s="1">
+        <v>0</v>
+      </c>
+      <c r="Z159" s="1">
+        <v>0</v>
+      </c>
+      <c r="AA159" s="1">
+        <v>0</v>
+      </c>
+      <c r="AB159" s="1">
+        <v>0</v>
+      </c>
+      <c r="AC159" s="1">
+        <v>0</v>
+      </c>
+      <c r="AD159" s="1">
+        <v>752</v>
+      </c>
+      <c r="AE159" s="1">
+        <v>58</v>
+      </c>
+      <c r="AF159" s="1">
+        <v>0</v>
+      </c>
+      <c r="AG159" s="1">
+        <v>27</v>
+      </c>
+      <c r="AH159" s="1">
+        <v>253</v>
+      </c>
+      <c r="AI159" s="1">
+        <v>0</v>
+      </c>
+      <c r="AJ159" s="1">
+        <v>10</v>
+      </c>
+      <c r="AK159" s="1">
+        <v>0</v>
+      </c>
+      <c r="AL159" s="1">
+        <v>0</v>
+      </c>
+      <c r="AM159" s="1">
+        <v>0</v>
+      </c>
+      <c r="AN159" s="1">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="160" spans="1:40" x14ac:dyDescent="0.25">
+      <c r="A160" s="10">
+        <v>45906</v>
+      </c>
+      <c r="B160" s="1">
+        <v>157</v>
+      </c>
+      <c r="C160" s="1">
+        <v>89</v>
+      </c>
+      <c r="D160" s="1">
+        <v>0</v>
+      </c>
+      <c r="E160" s="1">
+        <v>0</v>
+      </c>
+      <c r="F160" s="1">
+        <v>915</v>
+      </c>
+      <c r="G160" s="1">
+        <v>222</v>
+      </c>
+      <c r="H160" s="1">
+        <v>1</v>
+      </c>
+      <c r="I160" s="1">
+        <v>0</v>
+      </c>
+      <c r="J160" s="1"/>
+      <c r="K160" s="1">
+        <v>0</v>
+      </c>
+      <c r="L160" s="1">
+        <v>199</v>
+      </c>
+      <c r="M160" s="1">
+        <v>0</v>
+      </c>
+      <c r="N160" s="1">
+        <v>0</v>
+      </c>
+      <c r="O160" s="1">
+        <v>7</v>
+      </c>
+      <c r="P160" s="1">
+        <v>0</v>
+      </c>
+      <c r="Q160" s="1">
+        <v>0</v>
+      </c>
+      <c r="R160" s="1">
+        <v>120</v>
+      </c>
+      <c r="S160" s="1">
+        <v>37</v>
+      </c>
+      <c r="T160" s="1">
+        <v>0</v>
+      </c>
+      <c r="U160" s="1">
+        <v>73</v>
+      </c>
+      <c r="V160" s="1">
+        <v>16</v>
+      </c>
+      <c r="W160" s="1">
+        <v>0</v>
+      </c>
+      <c r="X160" s="1">
+        <v>0</v>
+      </c>
+      <c r="Y160" s="1">
+        <v>0</v>
+      </c>
+      <c r="Z160" s="1">
+        <v>0</v>
+      </c>
+      <c r="AA160" s="1">
+        <v>0</v>
+      </c>
+      <c r="AB160" s="1">
+        <v>0</v>
+      </c>
+      <c r="AC160" s="1">
+        <v>0</v>
+      </c>
+      <c r="AD160" s="1">
+        <v>864</v>
+      </c>
+      <c r="AE160" s="1">
+        <v>51</v>
+      </c>
+      <c r="AF160" s="1">
+        <v>0</v>
+      </c>
+      <c r="AG160" s="1">
+        <v>23</v>
+      </c>
+      <c r="AH160" s="1">
+        <v>199</v>
+      </c>
+      <c r="AI160" s="1">
+        <v>0</v>
+      </c>
+      <c r="AJ160" s="1">
+        <v>1</v>
+      </c>
+      <c r="AK160" s="1">
+        <v>0</v>
+      </c>
+      <c r="AL160" s="1">
+        <v>0</v>
+      </c>
+      <c r="AM160" s="1">
+        <v>0</v>
+      </c>
+      <c r="AN160" s="1">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="161" spans="1:40" x14ac:dyDescent="0.25">
+      <c r="A161" s="10">
+        <v>45907</v>
+      </c>
+      <c r="B161" s="1">
+        <v>494.5</v>
+      </c>
+      <c r="C161" s="1">
+        <v>82</v>
+      </c>
+      <c r="D161" s="1">
+        <v>0</v>
+      </c>
+      <c r="E161" s="1">
+        <v>0</v>
+      </c>
+      <c r="F161" s="1">
+        <v>1011.5</v>
+      </c>
+      <c r="G161" s="1">
+        <v>250.5</v>
+      </c>
+      <c r="H161" s="1">
+        <v>2</v>
+      </c>
+      <c r="I161" s="1">
+        <v>0</v>
+      </c>
+      <c r="J161" s="1"/>
+      <c r="K161" s="1">
+        <v>0</v>
+      </c>
+      <c r="L161" s="1">
+        <v>288</v>
+      </c>
+      <c r="M161" s="1">
+        <v>0</v>
+      </c>
+      <c r="N161" s="1">
+        <v>0</v>
+      </c>
+      <c r="O161" s="1">
+        <v>6.5</v>
+      </c>
+      <c r="P161" s="1">
+        <v>0</v>
+      </c>
+      <c r="Q161" s="1">
+        <v>0</v>
+      </c>
+      <c r="R161" s="1">
+        <v>295.5</v>
+      </c>
+      <c r="S161" s="1">
+        <v>199</v>
+      </c>
+      <c r="T161" s="1">
+        <v>0</v>
+      </c>
+      <c r="U161" s="1">
+        <v>69.5</v>
+      </c>
+      <c r="V161" s="1">
+        <v>12.5</v>
+      </c>
+      <c r="W161" s="1">
+        <v>0</v>
+      </c>
+      <c r="X161" s="1">
+        <v>0</v>
+      </c>
+      <c r="Y161" s="1">
+        <v>0</v>
+      </c>
+      <c r="Z161" s="1">
+        <v>0</v>
+      </c>
+      <c r="AA161" s="1">
+        <v>0</v>
+      </c>
+      <c r="AB161" s="1">
+        <v>0</v>
+      </c>
+      <c r="AC161" s="1">
+        <v>0</v>
+      </c>
+      <c r="AD161" s="1">
+        <v>954</v>
+      </c>
+      <c r="AE161" s="1">
+        <v>57.5</v>
+      </c>
+      <c r="AF161" s="1">
+        <v>0</v>
+      </c>
+      <c r="AG161" s="1">
+        <v>37.5</v>
+      </c>
+      <c r="AH161" s="1">
+        <v>213</v>
+      </c>
+      <c r="AI161" s="1">
+        <v>0</v>
+      </c>
+      <c r="AJ161" s="1">
+        <v>0.5</v>
+      </c>
+      <c r="AK161" s="1">
+        <v>1.5</v>
+      </c>
+      <c r="AL161" s="1">
+        <v>0</v>
+      </c>
+      <c r="AM161" s="1">
+        <v>0</v>
+      </c>
+      <c r="AN161" s="1">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="162" spans="1:40" x14ac:dyDescent="0.25">
+      <c r="A162" s="10">
+        <v>45908</v>
+      </c>
+      <c r="B162" s="1">
+        <v>832</v>
+      </c>
+      <c r="C162" s="1">
+        <v>75</v>
+      </c>
+      <c r="D162" s="1">
+        <v>0</v>
+      </c>
+      <c r="E162" s="1">
+        <v>0</v>
+      </c>
+      <c r="F162" s="1">
+        <v>1108</v>
+      </c>
+      <c r="G162" s="1">
+        <v>279</v>
+      </c>
+      <c r="H162" s="1">
+        <v>3</v>
+      </c>
+      <c r="I162" s="1">
+        <v>0</v>
+      </c>
+      <c r="J162" s="1"/>
+      <c r="K162" s="1">
+        <v>0</v>
+      </c>
+      <c r="L162" s="1">
+        <v>377</v>
+      </c>
+      <c r="M162" s="1">
+        <v>0</v>
+      </c>
+      <c r="N162" s="1">
+        <v>0</v>
+      </c>
+      <c r="O162" s="1">
+        <v>6</v>
+      </c>
+      <c r="P162" s="1">
+        <v>0</v>
+      </c>
+      <c r="Q162" s="1">
+        <v>0</v>
+      </c>
+      <c r="R162" s="1">
+        <v>471</v>
+      </c>
+      <c r="S162" s="1">
+        <v>361</v>
+      </c>
+      <c r="T162" s="1">
+        <v>0</v>
+      </c>
+      <c r="U162" s="1">
+        <v>66</v>
+      </c>
+      <c r="V162" s="1">
+        <v>9</v>
+      </c>
+      <c r="W162" s="1">
+        <v>0</v>
+      </c>
+      <c r="X162" s="1">
+        <v>0</v>
+      </c>
+      <c r="Y162" s="1">
+        <v>0</v>
+      </c>
+      <c r="Z162" s="1">
+        <v>0</v>
+      </c>
+      <c r="AA162" s="1">
+        <v>0</v>
+      </c>
+      <c r="AB162" s="1">
+        <v>0</v>
+      </c>
+      <c r="AC162" s="1">
+        <v>0</v>
+      </c>
+      <c r="AD162" s="1">
+        <v>1044</v>
+      </c>
+      <c r="AE162" s="1">
+        <v>64</v>
+      </c>
+      <c r="AF162" s="1">
+        <v>0</v>
+      </c>
+      <c r="AG162" s="1">
+        <v>52</v>
+      </c>
+      <c r="AH162" s="1">
+        <v>227</v>
+      </c>
+      <c r="AI162" s="1">
+        <v>0</v>
+      </c>
+      <c r="AJ162" s="1">
+        <v>0</v>
+      </c>
+      <c r="AK162" s="1">
+        <v>3</v>
+      </c>
+      <c r="AL162" s="1">
+        <v>0</v>
+      </c>
+      <c r="AM162" s="1">
+        <v>0</v>
+      </c>
+      <c r="AN162" s="1">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="163" spans="1:40" x14ac:dyDescent="0.25">
+      <c r="A163" s="10">
+        <v>45909</v>
+      </c>
+      <c r="B163" s="1">
+        <v>903</v>
+      </c>
+      <c r="C163" s="1">
+        <v>57</v>
+      </c>
+      <c r="D163" s="1">
+        <v>0</v>
+      </c>
+      <c r="E163" s="1">
+        <v>0</v>
+      </c>
+      <c r="F163" s="1">
+        <v>1125</v>
+      </c>
+      <c r="G163" s="1">
+        <v>201</v>
+      </c>
+      <c r="H163" s="1">
+        <v>12</v>
+      </c>
+      <c r="I163" s="1">
+        <v>0</v>
+      </c>
+      <c r="J163" s="1"/>
+      <c r="K163" s="1">
+        <v>0</v>
+      </c>
+      <c r="L163" s="1">
+        <v>585</v>
+      </c>
+      <c r="M163" s="1">
+        <v>0</v>
+      </c>
+      <c r="N163" s="1">
+        <v>0</v>
+      </c>
+      <c r="O163" s="1">
+        <v>6</v>
+      </c>
+      <c r="P163" s="1">
+        <v>0</v>
+      </c>
+      <c r="Q163" s="1">
+        <v>0</v>
+      </c>
+      <c r="R163" s="1">
+        <v>408</v>
+      </c>
+      <c r="S163" s="1">
+        <v>495</v>
+      </c>
+      <c r="T163" s="1">
+        <v>0</v>
+      </c>
+      <c r="U163" s="1">
+        <v>42</v>
+      </c>
+      <c r="V163" s="1">
         <v>15</v>
       </c>
-      <c r="AN157" s="1">
+      <c r="W163" s="1">
+        <v>0</v>
+      </c>
+      <c r="X163" s="1">
+        <v>0</v>
+      </c>
+      <c r="Y163" s="1">
+        <v>0</v>
+      </c>
+      <c r="Z163" s="1">
+        <v>0</v>
+      </c>
+      <c r="AA163" s="1">
+        <v>0</v>
+      </c>
+      <c r="AB163" s="1">
+        <v>0</v>
+      </c>
+      <c r="AC163" s="1">
+        <v>0</v>
+      </c>
+      <c r="AD163" s="1">
+        <v>987</v>
+      </c>
+      <c r="AE163" s="1">
+        <v>138</v>
+      </c>
+      <c r="AF163" s="1">
+        <v>0</v>
+      </c>
+      <c r="AG163" s="1">
+        <v>45</v>
+      </c>
+      <c r="AH163" s="1">
+        <v>156</v>
+      </c>
+      <c r="AI163" s="1">
+        <v>0</v>
+      </c>
+      <c r="AJ163" s="1">
+        <v>3</v>
+      </c>
+      <c r="AK163" s="1">
+        <v>9</v>
+      </c>
+      <c r="AL163" s="1">
+        <v>0</v>
+      </c>
+      <c r="AM163" s="1">
+        <v>0</v>
+      </c>
+      <c r="AN163" s="1">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="164" spans="1:40" x14ac:dyDescent="0.25">
+      <c r="A164" s="10"/>
+      <c r="B164" s="14">
+        <v>5115</v>
+      </c>
+      <c r="C164" s="14">
+        <v>1264.5</v>
+      </c>
+      <c r="D164" s="14">
+        <v>0</v>
+      </c>
+      <c r="E164" s="14">
+        <v>0</v>
+      </c>
+      <c r="F164" s="14">
+        <v>12133.5</v>
+      </c>
+      <c r="G164" s="14">
+        <v>3848</v>
+      </c>
+      <c r="H164" s="14">
+        <v>990</v>
+      </c>
+      <c r="I164" s="14">
+        <v>16</v>
+      </c>
+      <c r="J164" s="1"/>
+      <c r="K164" s="1">
+        <v>0</v>
+      </c>
+      <c r="L164" s="1">
+        <v>437170.96</v>
+      </c>
+      <c r="M164" s="1">
+        <v>0</v>
+      </c>
+      <c r="N164" s="1">
+        <v>0</v>
+      </c>
+      <c r="O164" s="1">
+        <v>3857.5</v>
+      </c>
+      <c r="P164" s="1">
+        <v>0</v>
+      </c>
+      <c r="Q164" s="1">
+        <v>0</v>
+      </c>
+      <c r="R164" s="1">
+        <v>3442.5</v>
+      </c>
+      <c r="S164" s="1">
+        <v>1672.5</v>
+      </c>
+      <c r="T164" s="1">
+        <v>0</v>
+      </c>
+      <c r="U164" s="1">
+        <v>1123</v>
+      </c>
+      <c r="V164" s="1">
+        <v>141.5</v>
+      </c>
+      <c r="W164" s="1">
+        <v>0</v>
+      </c>
+      <c r="X164" s="1">
+        <v>0</v>
+      </c>
+      <c r="Y164" s="1">
+        <v>0</v>
+      </c>
+      <c r="Z164" s="1">
+        <v>0</v>
+      </c>
+      <c r="AA164" s="1">
+        <v>0</v>
+      </c>
+      <c r="AB164" s="1">
+        <v>0</v>
+      </c>
+      <c r="AC164" s="1">
+        <v>0</v>
+      </c>
+      <c r="AD164" s="1">
+        <v>11052.5</v>
+      </c>
+      <c r="AE164" s="1">
+        <v>1081</v>
+      </c>
+      <c r="AF164" s="1">
+        <v>0</v>
+      </c>
+      <c r="AG164" s="1">
+        <v>620.5</v>
+      </c>
+      <c r="AH164" s="1">
+        <v>3227.5</v>
+      </c>
+      <c r="AI164" s="1">
+        <v>0</v>
+      </c>
+      <c r="AJ164" s="1">
+        <v>851.5</v>
+      </c>
+      <c r="AK164" s="1">
+        <v>138.5</v>
+      </c>
+      <c r="AL164" s="1">
+        <v>0</v>
+      </c>
+      <c r="AM164" s="1">
+        <v>15</v>
+      </c>
+      <c r="AN164" s="1">
         <v>1</v>
       </c>
     </row>
-    <row r="158" spans="1:40" x14ac:dyDescent="0.25">
-      <c r="A158" s="10"/>
-      <c r="B158" s="1"/>
-      <c r="C158" s="1"/>
-      <c r="D158" s="1"/>
-      <c r="E158" s="1"/>
-      <c r="F158" s="1"/>
-      <c r="G158" s="1"/>
-      <c r="H158" s="1"/>
-      <c r="I158" s="1"/>
-    </row>
-    <row r="159" spans="1:40" x14ac:dyDescent="0.25">
-      <c r="A159" s="10"/>
-      <c r="B159" s="1"/>
-      <c r="C159" s="1"/>
-      <c r="D159" s="1"/>
-      <c r="E159" s="1"/>
-      <c r="F159" s="1"/>
-      <c r="G159" s="1"/>
-      <c r="H159" s="1"/>
-      <c r="I159" s="1"/>
-    </row>
-    <row r="160" spans="1:40" x14ac:dyDescent="0.25">
-      <c r="A160" s="10"/>
-      <c r="B160" s="1"/>
-      <c r="C160" s="1"/>
-      <c r="D160" s="1"/>
-      <c r="E160" s="1"/>
-      <c r="F160" s="1"/>
-      <c r="G160" s="1"/>
-      <c r="H160" s="1"/>
-      <c r="I160" s="1"/>
-    </row>
-    <row r="161" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A161" s="10"/>
-      <c r="B161" s="1"/>
-      <c r="C161" s="1"/>
-      <c r="D161" s="1"/>
-      <c r="E161" s="1"/>
-      <c r="F161" s="1"/>
-      <c r="G161" s="1"/>
-      <c r="H161" s="1"/>
-      <c r="I161" s="1"/>
-    </row>
-    <row r="162" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A162" s="10"/>
-      <c r="B162" s="1"/>
-      <c r="C162" s="1"/>
-      <c r="D162" s="1"/>
-      <c r="E162" s="1"/>
-      <c r="F162" s="1"/>
-      <c r="G162" s="1"/>
-      <c r="H162" s="1"/>
-      <c r="I162" s="1"/>
-    </row>
-    <row r="163" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A163" s="10"/>
-      <c r="B163" s="1"/>
-      <c r="C163" s="1"/>
-      <c r="D163" s="1"/>
-      <c r="E163" s="1"/>
-      <c r="F163" s="1"/>
-      <c r="G163" s="1"/>
-      <c r="H163" s="1"/>
-      <c r="I163" s="1"/>
-    </row>
-    <row r="164" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A164" s="10"/>
-      <c r="B164" s="1"/>
-      <c r="C164" s="1"/>
-      <c r="D164" s="1"/>
-      <c r="E164" s="1"/>
-      <c r="F164" s="1"/>
-      <c r="G164" s="1"/>
-      <c r="H164" s="1"/>
-      <c r="I164" s="1"/>
-    </row>
-    <row r="165" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="165" spans="1:40" x14ac:dyDescent="0.25">
       <c r="A165" s="10"/>
       <c r="B165" s="1"/>
       <c r="C165" s="1"/>
@@ -41107,7 +42304,7 @@
       <c r="H165" s="1"/>
       <c r="I165" s="1"/>
     </row>
-    <row r="166" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="166" spans="1:40" x14ac:dyDescent="0.25">
       <c r="A166" s="10"/>
       <c r="B166" s="1"/>
       <c r="C166" s="1"/>
@@ -41118,7 +42315,7 @@
       <c r="H166" s="1"/>
       <c r="I166" s="1"/>
     </row>
-    <row r="167" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="167" spans="1:40" x14ac:dyDescent="0.25">
       <c r="A167" s="10"/>
       <c r="B167" s="1"/>
       <c r="C167" s="1"/>
@@ -41129,7 +42326,7 @@
       <c r="H167" s="1"/>
       <c r="I167" s="1"/>
     </row>
-    <row r="168" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="168" spans="1:40" x14ac:dyDescent="0.25">
       <c r="A168" s="10"/>
       <c r="B168" s="1"/>
       <c r="C168" s="1"/>
@@ -41140,7 +42337,7 @@
       <c r="H168" s="1"/>
       <c r="I168" s="1"/>
     </row>
-    <row r="169" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="169" spans="1:40" x14ac:dyDescent="0.25">
       <c r="A169" s="10"/>
       <c r="B169" s="1"/>
       <c r="C169" s="1"/>
@@ -41151,7 +42348,7 @@
       <c r="H169" s="1"/>
       <c r="I169" s="1"/>
     </row>
-    <row r="170" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="170" spans="1:40" x14ac:dyDescent="0.25">
       <c r="A170" s="10"/>
       <c r="B170" s="1"/>
       <c r="C170" s="1"/>
@@ -41162,7 +42359,7 @@
       <c r="H170" s="1"/>
       <c r="I170" s="1"/>
     </row>
-    <row r="171" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="171" spans="1:40" x14ac:dyDescent="0.25">
       <c r="A171" s="10"/>
       <c r="B171" s="1"/>
       <c r="C171" s="1"/>
@@ -41173,7 +42370,7 @@
       <c r="H171" s="1"/>
       <c r="I171" s="1"/>
     </row>
-    <row r="172" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="172" spans="1:40" x14ac:dyDescent="0.25">
       <c r="A172" s="10"/>
       <c r="B172" s="1"/>
       <c r="C172" s="1"/>
@@ -41184,7 +42381,7 @@
       <c r="H172" s="1"/>
       <c r="I172" s="1"/>
     </row>
-    <row r="173" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="173" spans="1:40" x14ac:dyDescent="0.25">
       <c r="A173" s="10"/>
       <c r="B173" s="1"/>
       <c r="C173" s="1"/>
@@ -41195,7 +42392,7 @@
       <c r="H173" s="1"/>
       <c r="I173" s="1"/>
     </row>
-    <row r="174" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="174" spans="1:40" x14ac:dyDescent="0.25">
       <c r="A174" s="10"/>
       <c r="B174" s="1"/>
       <c r="C174" s="1"/>
@@ -41206,7 +42403,7 @@
       <c r="H174" s="1"/>
       <c r="I174" s="1"/>
     </row>
-    <row r="175" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="175" spans="1:40" x14ac:dyDescent="0.25">
       <c r="A175" s="10"/>
       <c r="B175" s="1"/>
       <c r="C175" s="1"/>
@@ -41217,7 +42414,7 @@
       <c r="H175" s="1"/>
       <c r="I175" s="1"/>
     </row>
-    <row r="176" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="176" spans="1:40" x14ac:dyDescent="0.25">
       <c r="A176" s="10"/>
       <c r="B176" s="1"/>
       <c r="C176" s="1"/>

</xml_diff>